<commit_message>
Melhoria na base de dados para evitar nome de partidos no QUIZ
</commit_message>
<xml_diff>
--- a/planos_governo.xlsx
+++ b/planos_governo.xlsx
@@ -484,7 +484,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="120" customHeight="1">
+    <row r="2" ht="135" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>13</t>
@@ -507,12 +507,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>O programa prioriza a educação básica, com metas do Compromisso Nacional Criança Alfabetizada para chegar a 80% das crianças alfabetizadas na idade certa, e prevê expandir a educação em tempo integral com financiamento do Fundeb. Propõe dar continuidade ao Pé-de-Meia para combater a evasão no ensino médio, ampliar os Institutos Federais, o MEC Livros e o MEC Idiomas, além de universalizar a internet nas escolas. Também busca valorizar os professores, mantendo o Piso do Magistério, o Pé-de-Meia Licenciatura e o Bolsa Mais Professores. Por fim, prevê ampliar o financiamento do ensino superior e técnico, com novos campi, ProUni e FIES, cumprindo o Plano Nacional de Educação 2026-2036.</t>
+          <t>O programa prioriza a educação básica, com metas de alfabetização para chegar a 80% das crianças alfabetizadas na idade certa, e prevê expandir a educação em tempo integral com financiamento do Fundeb. Propõe dar continuidade a um incentivo financeiro mensal para alunos do ensino médio permanecerem na escola, ampliar os Institutos Federais e programas de distribuição de livros didáticos e de ensino gratuito de idiomas, além de universalizar a internet nas escolas. Também busca valorizar os professores, mantendo o piso salarial nacional do magistério e bolsas para formação e atração de novos docentes. Por fim, prevê ampliar o financiamento do ensino superior e técnico, com novos campi e bolsas e financiamento estudantil em universidades públicas e privadas, cumprindo as metas do plano nacional de educação para o período 2026-2036.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Mais creches, tempo integral, Pé-de-Meia contra evasão, alfabetização até os 80% e expansão de institutos federais e universidades.</t>
+          <t>Mais colégios em tempo integral, incentivo financeiro contra evasão escolar, 80% de alfabetização na idade certa e financiamento estudantil.</t>
         </is>
       </c>
     </row>
@@ -539,12 +539,12 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>O plano mantém o novo arcabouço fiscal e busca criar condições para reduzir os juros com inflação controlada, aliando responsabilidade fiscal a investimentos sociais. Aposta na neoindustrialização por meio da Nova Indústria Brasil (NIB), com foco em inteligência artificial, minerais críticos e soberania tecnológica. Prevê ampliar investimentos em infraestrutura logística pelo Novo PAC (rodovias, ferrovias, portos, aeroportos) e fortalecer a economia digital. Também propõe apoiar micro e pequenas empresas, com crédito via Pronampe e Procred 360, e promover o desenvolvimento regional equilibrado, valorizando a Amazônia e o Nordeste como polos estratégicos.</t>
+          <t>O plano mantém o novo arcabouço fiscal e busca criar condições para reduzir os juros com inflação controlada, aliando responsabilidade fiscal a investimentos sociais. Aposta em uma política de reindustrialização, com foco em inteligência artificial, minerais críticos e soberania tecnológica. Prevê ampliar investimentos em infraestrutura logística por meio de um amplo programa de obras (rodovias, ferrovias, portos, aeroportos) e fortalecer a economia digital. Também propõe apoiar micro e pequenas empresas, com linhas de crédito facilitado, e promover o desenvolvimento regional equilibrado, valorizando a Amazônia e o Nordeste como polos estratégicos.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Reformas fiscal e tributária, juros mais baixos, neoindustrialização (NIB) e investimentos recordes em infraestrutura pelo Novo PAC.</t>
+          <t>Reformas fiscal e tributária, juros mais baixos, reindustrialização com foco em IA e minerais críticos e investimentos em infraestrutura.</t>
         </is>
       </c>
     </row>
@@ -571,16 +571,16 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>O programa reafirma o compromisso com o SUS público e universal, ampliando a atenção básica, o Programa Mais Médicos, o Farmácia Popular e a integração digital dos dados de saúde, com prontuário único e telemedicina. Propõe reduzir as filas na atenção especializada por meio do Agora Tem Especialistas, expandir a maior rede pública de cuidado ao câncer do mundo e fortalecer a saúde da mulher, a saúde mental e a vacinação infantil. Busca também ampliar a soberania sanitária por meio do Complexo Econômico-Industrial da Saúde, produzindo insumos, vacinas e medicamentos no país.</t>
+          <t>O programa reafirma o compromisso com o SUS público e universal, ampliando a atenção básica, programas de provimento de médicos em regiões carentes, a distribuição gratuita de medicamentos e a integração digital dos dados de saúde, com prontuário único e telemedicina. Propõe reduzir as filas na atenção especializada por meio de mutirões de consultas e exames, expandir a maior rede pública de cuidado ao câncer do mundo e fortalecer a saúde da mulher, a saúde mental e a vacinação infantil. Busca também ampliar a soberania sanitária, produzindo insumos, vacinas e medicamentos no país.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>SUS mais forte: mais médicos, menos filas com o Agora Tem Especialistas, Farmácia Popular e soberania na produção de medicamentos.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="105" customHeight="1">
+          <t>SUS mais forte: mais médicos, menos filas com mutirões de especialistas, remédios gratuitos e soberania na produção de medicamentos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>13</t>
@@ -603,12 +603,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe criar o Ministério da Segurança Pública, aprovar a PEC da Segurança Pública e fortalecer o Sistema Único de Segurança Pública (SUSP) para melhorar a coordenação federativa. Prevê intensificar o combate ao crime organizado e às milícias com base na Lei Antifacção e na estratégia de asfixia financeira, além de manter o controle de armas de fogo. Propõe reforçar as Forças Integradas de Combate ao Crime Organizado (FICCOs) na Amazônia, modernizar o sistema prisional e ampliar o policiamento de proximidade e o uso de câmeras corporais. Também busca reforçar o combate a crimes cibernéticos e à violência contra mulheres, crianças e adolescentes.</t>
+          <t>O plano propõe criar o Ministério da Segurança Pública, aprovar a PEC da Segurança Pública e fortalecer o Sistema Único de Segurança Pública (SUSP) para melhorar a coordenação federativa. Prevê intensificar o combate ao crime organizado e às milícias com uma nova lei de combate a facções criminosas e a estratégia de asfixia financeira, além de manter o controle de armas de fogo. Propõe reforçar forças-tarefa integradas de combate ao crime organizado na Amazônia, modernizar o sistema prisional e ampliar o policiamento de proximidade e o uso de câmeras corporais. Também busca reforçar o combate a crimes cibernéticos e à violência contra mulheres, crianças e adolescentes.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Novo Ministério da Segurança Pública, Lei Antifacção contra o crime organizado, controle de armas e mais policiamento de proximidade.</t>
+          <t>Criar o Ministério da Segurança Pública, nova lei contra o crime organizado, controle de armas e mais policiamento de proximidade.</t>
         </is>
       </c>
     </row>
@@ -635,16 +635,16 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>O programa prevê continuar investindo em mobilidade urbana, com expansão de metrôs, trens, VLTs e corredores exclusivos de ônibus (BRT), além de renovar e eletrificar progressivamente as frotas de transporte coletivo. Na logística nacional, propõe dar sequência ao Novo PAC com novas concessões rodoviárias, ferroviárias, portuárias e investimentos em aeroportos regionais. Destaca a integração multimodal do transporte como forma de reduzir desigualdades regionais e dar mais competitividade à produção nacional, priorizando também a integração das regiões metropolitanas e das cidades médias.</t>
+          <t>O programa prevê continuar investindo em mobilidade urbana, com expansão de metrôs, trens, VLTs e corredores exclusivos de ônibus (BRT), além de renovar e eletrificar progressivamente as frotas de transporte coletivo. Na logística nacional, propõe dar sequência a um amplo programa de investimentos, com novas concessões rodoviárias, ferroviárias, portuárias e investimentos em aeroportos regionais. Destaca a integração multimodal do transporte como forma de reduzir desigualdades regionais e dar mais competitividade à produção nacional, priorizando também a integração das regiões metropolitanas e das cidades médias.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Mais metrôs, trens, VLTs, corredores de ônibus e frotas elétricas, além de rodovias, ferrovias e portos modernizados pelo Novo PAC.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="90" customHeight="1">
+          <t>Mais metrôs, trens, VLTs, corredores de ônibus e frotas elétricas, além de rodovias, ferrovias e portos modernizados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="105" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>13</t>
@@ -667,16 +667,16 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>O programa reafirma a meta de desmatamento líquido zero até 2030 e o cumprimento da nova NDC brasileira, que prevê redução de 59% a 67% das emissões de gases de efeito estufa até 2035. Propõe fortalecer o Plano Clima, o Fundo Amazônia, o Fundo Clima e o Fundo Florestas Tropicais para Sempre (TFFF), além de ampliar as unidades de conservação e a restauração florestal. Também prevê políticas de proteção animal, adaptação climática nas cidades e no semiárido, e a continuidade da liderança brasileira nas negociações climáticas internacionais, como a COP30.</t>
+          <t>O programa reafirma a meta de desmatamento líquido zero até 2030 e o cumprimento da nova NDC brasileira, que prevê redução de 59% a 67% das emissões de gases de efeito estufa até 2035. Propõe fortalecer um plano nacional de enfrentamento à mudança do clima e fundos nacionais e internacionais de financiamento climático e de conservação florestal, além de ampliar as unidades de conservação e a restauração florestal. Também prevê políticas de proteção animal, adaptação climática nas cidades e no semiárido, e a continuidade da liderança brasileira nas negociações climáticas internacionais, como a COP30.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Meta de desmatamento zero até 2030, nova NDC de redução de emissões e fortalecimento do Fundo Amazônia e do Fundo Clima.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="105" customHeight="1">
+          <t>Meta de desmatamento zero até 2030, nova NDC de redução de emissões e fortalecimento de fundos de proteção da Amazônia e do clima.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>13</t>
@@ -699,12 +699,12 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>O plano dá continuidade ao Bolsa Família, à valorização do salário-mínimo e à nova Política Nacional de Cuidados (Cuidotecas, cozinhas solidárias, lavanderias públicas), com foco em reduzir as desigualdades sociais e raciais. Prevê ampliar políticas para povos indígenas, quilombolas, mulheres (Pacto de Enfrentamento ao Feminicídio), pessoas idosas e pessoas com deficiência, além de garantir direitos à população LGBTQIAP+. Também busca fortalecer o SUAS e as políticas de proteção à infância e à juventude, incluindo o combate à pobreza infantil e a saúde mental de jovens.</t>
+          <t>O plano dá continuidade a um programa de transferência de renda para famílias em vulnerabilidade, à valorização do salário-mínimo e a uma nova política nacional de cuidados, com equipamentos comunitários como espaços de cuidado infantil, cozinhas solidárias e lavanderias públicas, com foco em reduzir as desigualdades sociais e raciais. Prevê ampliar políticas para povos indígenas, quilombolas e mulheres, com um pacto nacional de combate à violência contra as mulheres, além de políticas para pessoas idosas e pessoas com deficiência e para garantir direitos à população LGBTQIAP+. Também busca fortalecer o SUAS e as políticas de proteção à infância e à juventude, incluindo o combate à pobreza infantil e a saúde mental de jovens.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Bolsa Família, valorização do salário mínimo, política de cuidados e proteção a mulheres, idosos, povos indígenas e quilombolas.</t>
+          <t>Transferência de renda, valorização do salário mínimo, política de cuidados e proteção a mulheres, idosos, indígenas e quilombolas.</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>O programa defende a soberania nacional e o protagonismo do Brasil no cenário internacional, priorizando a integração sul-americana por meio do Mercosul e a Amazônia como eixo estratégico regional. Propõe fortalecer o BRICS, o G20, a cooperação Sul-Sul e as reformas da ONU, do FMI e da OMC em busca de uma ordem mundial mais justa e multilateral. Também prevê fortalecer as Forças Armadas e a indústria nacional de defesa, ampliar acordos comerciais e manter a liderança na diplomacia climática, dando continuidade a iniciativas como a Aliança Global contra a Fome e a Pobreza.</t>
+          <t>O programa defende a soberania nacional e o protagonismo do Brasil no cenário internacional, priorizando a integração sul-americana por meio do Mercosul e a Amazônia como eixo estratégico regional. Propõe fortalecer o BRICS, o G20, a cooperação Sul-Sul e as reformas da ONU, do FMI e da OMC em busca de uma ordem mundial mais justa e multilateral. Também prevê fortalecer as Forças Armadas e a indústria nacional de defesa, ampliar acordos comerciais e manter a liderança na diplomacia climática, dando continuidade a iniciativas internacionais de combate à fome e à pobreza.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>O plano busca fortalecer a soberania digital do Brasil, com investimentos em inteligência artificial nacional, supercomputadores soberanos e modelos de linguagem em português apoiados em uma plataforma nacional de dados. Propõe ampliar o FNDCT e o Programa Conhecimento Brasil para repatriar e fixar cientistas, integrando ciência, tecnologia e inovação à política industrial da Nova Indústria Brasil. Também prevê expandir a conectividade (5G e fibra óptica) e criar o Centro Nacional de Transparência Algorítmica para regular decisões automatizadas e o uso de IA.</t>
+          <t>O plano busca fortalecer a soberania digital do Brasil, com investimentos em inteligência artificial nacional, supercomputadores soberanos e modelos de linguagem em português apoiados em uma plataforma nacional de dados. Propõe ampliar o financiamento à ciência e tecnologia e criar um programa de repatriação e fixação de cientistas brasileiros, integrando ciência, tecnologia e inovação a uma política de reindustrialização. Também prevê expandir a conectividade (5G e fibra óptica) e criar um órgão nacional para regular decisões automatizadas e o uso de IA.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>O programa dá continuidade à valorização do salário-mínimo, defende a aprovação do fim da escala 6x1 e a redução da jornada para 40 horas sem perda salarial, e busca combater a pejotização espúria e a precarização do trabalho em plataformas digitais. Prevê fortalecer a Economia Popular e Solidária, o empreendedorismo e o cooperativismo, além de ampliar a igualdade salarial entre homens e mulheres. Na previdência, propõe reduzir as filas do INSS, modernizar os serviços previdenciários e criar mecanismos contributivos mais flexíveis para trabalhadores com trajetórias descontínuas.</t>
+          <t>O programa dá continuidade à valorização do salário-mínimo, defende a aprovação do fim da escala 6x1 e a redução da jornada para 40 horas sem perda salarial, e busca combater a pejotização espúria e a precarização do trabalho em plataformas digitais. Prevê fortalecer a economia popular e solidária, o empreendedorismo e o cooperativismo, além de ampliar a igualdade salarial entre homens e mulheres. Na previdência, propõe reduzir as filas do INSS, modernizar os serviços previdenciários e criar mecanismos contributivos mais flexíveis para trabalhadores com trajetórias descontínuas.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe aprofundar a participação social por meio de conferências e do orçamento participativo, além de modernizar o Estado com serviços públicos digitais personalizados via Gov.br e uma nova Política Nacional de Letramento Digital. Prevê fortalecer o combate à corrupção com o Plano de Integridade 2025-2027 e ampliar a transparência, usando inteligência artificial no Portal da Transparência. Também propõe debater a reforma do sistema de emendas parlamentares e aprimorar a cooperação federativa e o uso do poder de compra do Estado para o desenvolvimento dos territórios.</t>
+          <t>O plano propõe aprofundar a participação social por meio de conferências e do orçamento participativo, além de modernizar o Estado com serviços públicos digitais personalizados via Gov.br e uma nova política nacional de letramento digital. Prevê fortalecer o combate à corrupção com um plano de integridade para os próximos anos e ampliar a transparência, usando inteligência artificial no portal de transparência do governo. Também propõe debater a reforma do sistema de emendas parlamentares e aprimorar a cooperação federativa e o uso do poder de compra do Estado para o desenvolvimento dos territórios.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -836,7 +836,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="90" customHeight="1">
+    <row r="13" ht="120" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>13</t>
@@ -859,12 +859,12 @@
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>O programa prevê ampliar o Plano Safra da Agricultura Familiar e o Pronaf, fortalecer o PAA e a assistência técnica rural (ATER), além de incentivar a agroecologia e a produção orgânica pelo PLANAPO. Propõe continuar a reforma agrária, a regularização fundiária e a titulação de territórios quilombolas, junto com programas de acesso à água (Cisternas) e energia no campo. Para o agronegócio, busca ampliar o crédito rural, a rastreabilidade da pecuária, a modernização via Embrapa e a diversificação de mercados de exportação, mantendo o Brasil fora do Mapa da Fome.</t>
+          <t>O programa prevê ampliar o programa anual de crédito rural para a agricultura familiar e a linha de crédito federal para pequenos produtores, fortalecer o programa de compra de alimentos da agricultura familiar e a assistência técnica rural (ATER), além de incentivar a agroecologia e a produção orgânica por meio de um plano nacional de agroecologia. Propõe continuar a reforma agrária, a regularização fundiária e a titulação de territórios quilombolas, junto com programas de acesso à água e energia no campo. Para o agronegócio, busca ampliar o crédito rural, a rastreabilidade da pecuária, a modernização via Embrapa e a diversificação de mercados de exportação, mantendo o Brasil fora do Mapa da Fome.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Ampliação do Plano Safra e do Pronaf, reforma agrária, agroecologia e apoio ao agronegócio para manter o Brasil fora do Mapa da Fome.</t>
+          <t>Mais crédito rural para a agricultura familiar, reforma agrária, agroecologia e apoio ao agronegócio contra a fome no Brasil.</t>
         </is>
       </c>
     </row>
@@ -923,12 +923,12 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>O plano parte de um diagnóstico de crise fiscal crônica (dívida pública em R$8,64 tri, déficit crescente) e propõe uma PEC de Transição inspirada na "PEC do Equilíbrio Fiscal", desindexando benefícios do salário mínimo, desvinculando pisos de saúde e educação da receita e cortando isenções fiscais, com economia estimada de R$1,1 trilhão até 2031. Paralelamente, ataca a estagnação da produtividade nacional com reformas tributária, trabalhista, regulatória e de governança, além de substituir o Bolsa Família pelas "Frentes Cidadãs", programa de trabalho remunerado para beneficiários aptos. O objetivo declarado é liberar espaço fiscal para investimento e reduzir a carga tributária, encerrando o modelo de captura estatal e assistencialismo que hoje consome trilhões em subsídios.</t>
+          <t>O plano parte de um diagnóstico de crise fiscal crônica (dívida pública em R$8,64 tri, déficit crescente) e propõe uma PEC de Transição voltada ao equilíbrio fiscal, desindexando benefícios do salário mínimo, desvinculando pisos de saúde e educação da receita e cortando isenções fiscais, com economia estimada de R$1,1 trilhão até 2031. Paralelamente, ataca a estagnação da produtividade nacional com reformas tributária, trabalhista, regulatória e de governança, além de substituir o principal programa de transferência de renda por um novo programa de trabalho remunerado para beneficiários aptos. O objetivo declarado é liberar espaço fiscal para investimento e reduzir a carga tributária, encerrando o modelo de captura estatal e assistencialismo que hoje consome trilhões em subsídios.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Ajuste fiscal severo (PEC do Equilíbrio Fiscal) e fim do Bolsa Família, substituído por frentes de trabalho remuneradas.</t>
+          <t>Ajuste fiscal severo com nova PEC de equilíbrio fiscal e fim do programa de renda atual, substituído por frentes de trabalho remuneradas.</t>
         </is>
       </c>
     </row>
@@ -955,16 +955,16 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>O capítulo "SUS Fila Zero" propõe substituir a fila cronológica de atendimento por uma fila de prioridade de risco (ENER), baseada em gravidade clínica, risco de progressão e vulnerabilidade social. Prevê a criação do PRONTO, prontuário eletrônico nacional interoperável integrando atenção primária, hospitais, laboratórios e farmácias, além de um sistema digital de saúde com telemedicina e IA inspirado no DoctorSV de El Salvador. Também propõe integrar o Genomas Brasil ao prontuário, criar o Fundo Nacional de Modernização do Acesso com repasses condicionados a desempenho e adotar o modelo Hub-and-Spoke para concentrar casos complexos em centros regionais.</t>
+          <t>O plano de saúde propõe substituir a fila cronológica de atendimento por uma fila de prioridade de risco (ENER), baseada em gravidade clínica, risco de progressão e vulnerabilidade social. Prevê a criação de um prontuário eletrônico nacional interoperável, integrando atenção primária, hospitais, laboratórios e farmácias, além de um sistema digital de saúde com telemedicina e IA inspirado em experiências como a de El Salvador. Também propõe integrar o Genomas Brasil ao prontuário, criar um fundo nacional de modernização do acesso com repasses condicionados a desempenho e adotar o modelo Hub-and-Spoke para concentrar casos complexos em centros regionais.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>SUS Fila Zero: fila por risco clínico (ENER), prontuário nacional único (PRONTO), telemedicina e IA inspirados no modelo salvadorenho.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="105" customHeight="1">
+          <t>Saúde: fila por risco clínico (ENER), prontuário nacional único, telemedicina e IA inspirados em experiências como a salvadorenha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="120" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>14</t>
@@ -987,12 +987,12 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>O plano declara "Guerra ao Crime" contra facções como PCC e Comando Vermelho, adotando o Direito Penal do Inimigo (DPI) como marco jurídico, com decretação de Estado de Defesa, uma Lei Antifacção que permite banimento judicial de organizações criminosas, inversão do ônus da prova no confisco de bens e restrição de direitos a faccionados comprovados. Prevê intervenção federal e uso das Forças Armadas via GLO em territórios dominados, superpresídios de segurança máxima no modelo do CECOT salvadorenho, e investimento em tecnologia (scanners, drones, reconhecimento facial) para o combate ao crime organizado e à criminalidade urbana cotidiana.</t>
+          <t>O plano declara um combate frontal ao crime organizado, incluindo facções como PCC e Comando Vermelho, adotando o Direito Penal do Inimigo (DPI) como marco jurídico, com decretação de Estado de Defesa, uma lei antifacção que permite banimento judicial de organizações criminosas, inversão do ônus da prova no confisco de bens e restrição de direitos a faccionados comprovados. Prevê intervenção federal e uso das Forças Armadas via GLO em territórios dominados, superpresídios de segurança máxima no modelo do CECOT salvadorenho, e investimento em tecnologia (scanners, drones, reconhecimento facial) para o combate ao crime organizado e à criminalidade urbana cotidiana.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Guerra ao Crime desde o dia 1: Direito Penal do Inimigo contra facções, Lei Antifacção, GLO, e superpresídios no modelo CECOT salvadorenho.</t>
+          <t>Combate total ao crime desde o dia 1: Direito Penal do Inimigo contra facções, lei antifacção, GLO e superpresídios no modelo CECOT.</t>
         </is>
       </c>
     </row>
@@ -1019,12 +1019,12 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>O programa "Missão Rondon" busca elevar o investimento em infraestrutura dos atuais 2% para 4% do PIB, priorizando a expansão da malha ferroviária de 30 mil para ao menos 40 mil km (com obras como Ferrogrão, FIOL e Ferrovia Transoceânica), a ampliação de portos no Norte e Nordeste (Alcântara, Ilhéus, Itaqui) e aeroportos regionais. Propõe destravar o licenciamento ambiental para acelerar obras paralisadas (mais de 11 mil no país), mobilizar capital privado via concessões e PPPs e criar um novo regime de autorização ferroviária, além de reformar as licitações e capacitar órgãos técnicos municipais.</t>
+          <t>O plano de infraestrutura busca elevar o investimento dos atuais 2% para 4% do PIB, priorizando a expansão da malha ferroviária de 30 mil para ao menos 40 mil km (com obras como Ferrogrão, FIOL e Ferrovia Transoceânica), a ampliação de portos no Norte e Nordeste (Alcântara, Ilhéus, Itaqui) e aeroportos regionais. Propõe destravar o licenciamento ambiental para acelerar obras paralisadas (mais de 11 mil no país), mobilizar capital privado via concessões e PPPs e criar um novo regime de autorização ferroviária, além de reformar as licitações e capacitar órgãos técnicos municipais.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Missão Rondon: dobrar investimento em infraestrutura (2% para 4% do PIB), ampliar ferrovias para 40 mil km e destravar obras paralisadas.</t>
+          <t>Infraestrutura: dobrar investimento (2% para 4% do PIB), ampliar ferrovias para 40 mil km e destravar obras paralisadas.</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="105" customHeight="1">
+    <row r="20" ht="120" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>14</t>
@@ -1083,12 +1083,12 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>O eixo central da agenda social é a "desfavelização integral do Brasil em dez anos", transformando as 12.348 favelas do país (16,4 milhões de moradores) em bairros formais, com títulos de propriedade individual, regularização fundiária, serviços públicos obrigatórios (posto policial, escola, clínica, creche) e inserção de classe média para mistura social. O financiamento viria de um "título de desfavelização" com parcelas mensais subsidiadas, custando entre R$1,2 e R$1,5 trilhão em dez anos. Complementarmente, o plano substitui o Bolsa Família pelas "Frentes Cidadãs", programa de frentes de trabalho remuneradas para inserir beneficiários no mercado formal.</t>
+          <t>O eixo central da agenda social é a desfavelização integral do Brasil em dez anos, transformando as 12.348 favelas do país (16,4 milhões de moradores) em bairros formais, com títulos de propriedade individual, regularização fundiária, serviços públicos obrigatórios (posto policial, escola, clínica, creche) e inserção de classe média para mistura social. O financiamento viria de um título de desfavelização com parcelas mensais subsidiadas, custando entre R$1,2 e R$1,5 trilhão em dez anos. Complementarmente, o plano substitui o principal programa de transferência de renda por um novo programa de frentes de trabalho remuneradas para inserir beneficiários no mercado formal.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Desfavelização integral em 10 anos: favelas viram bairros formais com título de propriedade; Bolsa Família vira frentes de trabalho.</t>
+          <t>Desfavelização integral em 10 anos: favelas viram bairros formais com título de propriedade; renda básica vira frentes de trabalho.</t>
         </is>
       </c>
     </row>
@@ -1115,12 +1115,12 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>O plano "Brasil Poderoso" propõe uma doutrina de política externa pragmática, buscando posicionar o Brasil como "árbitro do Sul Global" na África, Ásia e América Latina, liderar um Pacto Interamericano contra o narcotráfico ancorado na OEA, promover a integração dos países lusófonos e uma "sub-hegemonia" sul-americana sem imperialismo. Defende a desdolarização regional com uma cesta de moedas liderada pelo real, uma postura pragmática dentro do BRICS+ diante da dominância chinesa, o fortalecimento da Base Industrial de Defesa e a busca da autonomia completa do ciclo de combustível nuclear como ativo estratégico de dissuasão.</t>
+          <t>O plano propõe uma doutrina de política externa pragmática, buscando posicionar o Brasil como árbitro do Sul Global na África, Ásia e América Latina, liderar um Pacto Interamericano contra o narcotráfico ancorado na OEA, promover a integração dos países lusófonos e uma sub-hegemonia sul-americana sem imperialismo. Defende a desdolarização regional com uma cesta de moedas liderada pelo real, uma postura pragmática dentro do BRICS+ diante da dominância chinesa, o fortalecimento da base industrial de defesa e a busca da autonomia completa do ciclo de combustível nuclear como ativo estratégico de dissuasão.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Brasil Poderoso: liderança no Sul Global, guerra ao narcotráfico via OEA, desdolarização regional com o real e domínio do ciclo nuclear.</t>
+          <t>Política externa pragmática: liderança no Sul Global, guerra ao narcotráfico via OEA, desdolarização com o real e domínio do ciclo nuclear.</t>
         </is>
       </c>
     </row>
@@ -1147,12 +1147,12 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>O plano cria o Marco Brasileiro da Inteligência Artificial (MBIA), com 14 medidas em cinco eixos que vão da redução de impostos e incentivo a venture capital para empresas de tecnologia, passando pela retenção e repatriação de talentos, até a instalação de datacenters para tornar o Brasil grande exportador de "inferência computacional" no Nordeste. Propõe o Projeto Abaporu, um laboratório nacional de IA com capital privado majoritário, e as Zonas Econômicas de Alta Inteligência (ZEAIs), além de integrar dados agropecuários na "Base Agro-Bio Nacional". Também investe pesado no domínio científico e industrial das terras raras, com planta-piloto de refino e centros de P&amp;D voltados à cadeia produtiva completa.</t>
+          <t>O plano cria um novo marco regulatório para a inteligência artificial, com 14 medidas em cinco eixos que vão da redução de impostos e incentivo a venture capital para empresas de tecnologia, passando pela retenção e repatriação de talentos, até a instalação de datacenters para tornar o Brasil grande exportador de inferência computacional no Nordeste. Propõe um laboratório nacional de IA com capital privado majoritário e zonas econômicas especiais voltadas a tecnologia de alta intensidade, além de integrar dados agropecuários em uma base nacional unificada. Também investe pesado no domínio científico e industrial das terras raras, com planta-piloto de refino e centros de P&amp;D voltados à cadeia produtiva completa.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Marco Brasileiro de IA (MBIA): incentivo a datacenters e venture capital, retenção de talentos e criação do Projeto Abaporu.</t>
+          <t>IA: novo marco regulatório com incentivo a datacenters e venture capital, retenção de talentos e um laboratório nacional de IA.</t>
         </is>
       </c>
     </row>
@@ -1179,12 +1179,12 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>O plano prevê a desindexação dos benefícios previdenciários e assistenciais do salário mínimo (corrigindo-os apenas pela inflação) como parte do ajuste fiscal, projetando economia de R$455 bilhões até 2031 só com essa medida, além de sinalizar a necessidade de reformar a previdência para viabilizar o equilíbrio das contas. Na frente trabalhista, defende a flexibilização das relações de trabalho e o enfrentamento da litigiosidade excessiva da Justiça do Trabalho como parte da agenda de produtividade. Também substitui o Bolsa Família pelo programa "Frentes Cidadãs", frentes de trabalho remuneradas voltadas à inserção da população economicamente ativa no mercado formal.</t>
+          <t>O plano prevê a desindexação dos benefícios previdenciários e assistenciais do salário mínimo (corrigindo-os apenas pela inflação) como parte do ajuste fiscal, projetando economia de R$455 bilhões até 2031 só com essa medida, além de sinalizar a necessidade de reformar a previdência para viabilizar o equilíbrio das contas. Na frente trabalhista, defende a flexibilização das relações de trabalho e o enfrentamento da litigiosidade excessiva da Justiça do Trabalho como parte da agenda de produtividade. Também substitui o principal programa de transferência de renda por frentes de trabalho remuneradas voltadas à inserção da população economicamente ativa no mercado formal.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Desindexação da Previdência do salário mínimo, flexibilização trabalhista e fim do Bolsa Família, substituído por frentes de trabalho.</t>
+          <t>Desindexação da Previdência do salário mínimo, flexibilização trabalhista e fim da renda básica atual, trocada por trabalho remunerado.</t>
         </is>
       </c>
     </row>
@@ -1211,12 +1211,12 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe a "Grande Consolidação Municipal", reduzindo o número de municípios de 5.570 para cerca de 1.656 conforme critérios de viabilidade fiscal, geográfica, econômica e urbana, acabando com duplicidades administrativas. Cria também a Lei de Responsabilidade Gerencial, com um Comissariado Federal de Gestão Pública que fiscaliza prefeituras em tempo real, condiciona repasses de fundos partidário e eleitoral ao desempenho dos gestores, permite intervenção federal (Tutela Gerencial) em municípios mal geridos e prevê a "Cláusula Antimáfia" para dissolver administrações capturadas pelo crime organizado, com gestão federal temporária de até 24 meses.</t>
+          <t>O plano propõe uma grande consolidação municipal, reduzindo o número de municípios de 5.570 para cerca de 1.656 conforme critérios de viabilidade fiscal, geográfica, econômica e urbana, acabando com duplicidades administrativas. Cria também uma lei de responsabilidade gerencial, com um órgão federal de gestão pública que fiscaliza prefeituras em tempo real, condiciona repasses de fundos partidário e eleitoral ao desempenho dos gestores, permite intervenção federal em municípios mal geridos e prevê um mecanismo para dissolver administrações capturadas pelo crime organizado, com gestão federal temporária de até 24 meses.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Grande Consolidação Municipal (5.570 para 1.656 municípios) e Lei de Responsabilidade Gerencial, que condiciona verbas a boa gestão.</t>
+          <t>Consolidação municipal (de 5.570 para 1.656 municípios) e lei de responsabilidade gerencial, que condiciona verbas a boa gestão.</t>
         </is>
       </c>
     </row>
@@ -1243,12 +1243,12 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>O programa "AgroBrasil 2030" assenta-se em cinco pilares: fim das invasões de propriedades rurais com endurecimento penal do esbulho possessório; auditoria e "produtivização" dos 140 milhões de hectares já destinados à reforma agrária, sem criação de novos assentamentos até que os existentes atinjam metas de produtividade; busca da soberania em fertilizantes, hoje 85% importados, com meta de reduzir essa dependência até 2035; incentivo à agroindústria e verticalização de cadeias produtivas (replicando o modelo do suco de laranja) via Zonas Econômicas Especiais e crédito do BNDES; e correção da narrativa educacional sobre o agronegócio, com auditoria de materiais didáticos em parceria com a Embrapa.</t>
+          <t>O plano para o agronegócio assenta-se em cinco pilares: fim das invasões de propriedades rurais com endurecimento penal do esbulho possessório; auditoria e produtivização dos 140 milhões de hectares já destinados à reforma agrária, sem criação de novos assentamentos até que os existentes atinjam metas de produtividade; busca da soberania em fertilizantes, hoje 85% importados, com meta de reduzir essa dependência até 2035; incentivo à agroindústria e verticalização de cadeias produtivas (replicando o modelo do suco de laranja) via zonas econômicas especiais e crédito do BNDES; e correção da narrativa educacional sobre o agronegócio, com auditoria de materiais didáticos em parceria com a Embrapa.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>AgroBrasil 2030: fim das invasões de terras, produtivização de assentamentos, soberania em fertilizantes e verticalização do agro.</t>
+          <t>Agro: fim das invasões de terras, produtivização de assentamentos, soberania em fertilizantes e verticalização das cadeias produtivas.</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>O programa defende educação pública, gratuita e de qualidade em todos os níveis, sem participação de empresas e fundações privadas na definição das políticas educacionais. Propõe fim das Parcerias Público-Privadas, das terceirizações e da compra de materiais dessas empresas pelas redes públicas, além da revogação da BNCC e do Novo Ensino Médio. Rejeita a militarização das escolas, projetos como Escola Sem Partido e a plataformização do ensino, defendendo uma formação crítica e científica. Propõe valorização dos profissionais da educação com carreira e salários dignos, ampliação de vagas em creches, escolas e universidades públicas, garantia de permanência estudantil e investimento massivo na educação pública, com um sistema único de ensino para todas as crianças e adolescentes.</t>
+          <t>O programa defende educação pública, gratuita e de qualidade em todos os níveis, sem participação de empresas e fundações privadas na definição das políticas educacionais. Propõe fim das Parcerias Público-Privadas, das terceirizações e da compra de materiais dessas empresas pelas redes públicas, além da revogação da BNCC e do Novo Ensino Médio. Rejeita a militarização das escolas, iniciativas de censura ao conteúdo escolar e a plataformização do ensino, defendendo uma formação crítica e científica. Propõe valorização dos profissionais da educação com carreira e salários dignos, ampliação de vagas em creches, escolas e universidades públicas, garantia de permanência estudantil e investimento massivo na educação pública, com um sistema único de ensino para todas as crianças e adolescentes.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1476,7 +1476,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="120" customHeight="1">
+    <row r="33" ht="135" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>16</t>
@@ -1499,12 +1499,12 @@
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>O documento defende romper com o imperialismo como condição para a soberania nacional, criticando tanto a submissão do governo Lula às potências capitalistas quanto o projeto de Flávio Bolsonaro de entregar a administração do país aos EUA após o tarifaço de Trump. Questiona também acordos como Mercosul-União Europeia e o avanço de fusões chinesas sobre setores estratégicos, considerando que nenhuma potência é alternativa real ao imperialismo. Defende que apenas a classe trabalhadora, organizada e em luta, pode enfrentar o grande capital internacional e conquistar real soberania, incluindo o controle nacional das riquezas como as terras raras. Aponta a luta anti-imperialista como parte de uma perspectiva de revolução latino-americana e internacional.</t>
+          <t>O documento defende romper com o imperialismo como condição para a soberania nacional, criticando tanto a submissão do governo atual às potências capitalistas quanto propostas de setores da oposição de entregar a administração do país a potências estrangeiras, especialmente após o recente tarifaço imposto por líderes estrangeiros. Questiona também acordos como Mercosul-União Europeia e o avanço de fusões chinesas sobre setores estratégicos, considerando que nenhuma potência é alternativa real ao imperialismo. Defende que apenas a classe trabalhadora, organizada e em luta, pode enfrentar o grande capital internacional e conquistar real soberania, incluindo o controle nacional das riquezas como as terras raras. Aponta a luta anti-imperialista como parte de uma perspectiva de revolução latino-americana e internacional.</t>
         </is>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Romper com o imperialismo: contra o tarifaço de Trump, a entrega do país aos EUA e a submissão de Lula às potências.</t>
+          <t>Romper com o imperialismo: contra o tarifaço estrangeiro, a entrega do país aos EUA e a submissão às grandes potências.</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="120" customHeight="1">
+    <row r="35" ht="135" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>16</t>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe fim da escala 6x1 sem redução de salário, redução da jornada de trabalho para 36 horas rumo à escala móvel e pleno emprego, aumento de 100% no salário mínimo e bolsa desemprego equivalente a um salário mínimo. Defende revogação da reforma trabalhista, da lei das terceirizações e da reforma da Previdência, com incorporação de terceirizados ao quadro efetivo via concurso público. Para trabalhadores de aplicativos, propõe reconhecimento do vínculo empregatício, direitos previdenciários plenos e transparência dos algoritmos, rejeitando o PLP 152. Na previdência, defende sistema público, solidário e universal, com redução da idade mínima de aposentadoria e inclusão de trabalhadores informais na proteção previdenciária.</t>
+          <t>O plano propõe fim da escala 6x1 sem redução de salário, redução da jornada de trabalho para 36 horas rumo à escala móvel e pleno emprego, aumento de 100% no salário mínimo e bolsa desemprego equivalente a um salário mínimo. Defende revogação da reforma trabalhista, da lei das terceirizações e da reforma da Previdência, com incorporação de terceirizados ao quadro efetivo via concurso público. Para trabalhadores de aplicativos, propõe reconhecimento do vínculo empregatício, direitos previdenciários plenos e transparência dos algoritmos, rejeitando o projeto de lei que mantém a terceirização desses trabalhadores. Na previdência, defende sistema público, solidário e universal, com redução da idade mínima de aposentadoria e inclusão de trabalhadores informais na proteção previdenciária.</t>
         </is>
       </c>
       <c r="F35" s="4" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>O programa propõe a nacionalização e estatização do sistema monetário e financeiro, com criação do Banco dos Trabalhadores e retomada do controle do Banco Central, revogando sua autonomia. Defende a reestruturação da dívida pública, com investigação de sua origem e suspensão temporária de juros. Propõe retomar empresas estratégicas privatizadas, controle do câmbio e comércio exterior, e uma reforma tributária progressiva com isenção para quem ganha até um salário-mínimo. Também prevê revogação do Arcabouço Fiscal e da Lei de Responsabilidade Fiscal e uma nova política industrial voltada à soberania tecnológica.</t>
+          <t>O programa propõe a nacionalização e estatização do sistema monetário e financeiro, com criação de um banco público voltado aos trabalhadores e retomada do controle do Banco Central, revogando sua autonomia. Defende a reestruturação da dívida pública, com investigação de sua origem e suspensão temporária de juros. Propõe retomar empresas estratégicas privatizadas, controle do câmbio e comércio exterior, e uma reforma tributária progressiva com isenção para quem ganha até um salário-mínimo. Também prevê revogação das atuais regras fiscais e da Lei de Responsabilidade Fiscal, além de uma nova política industrial voltada à soberania tecnológica.</t>
         </is>
       </c>
       <c r="F39" s="4" t="inlineStr">
@@ -1732,7 +1732,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="105" customHeight="1">
+    <row r="41" ht="120" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
           <t>21</t>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe uma política de segurança dos direitos no lugar da atual segurança pública, com desmilitarização completa, unificação das polícias e ciclo completo de formação. Defende o fim da política de guerra às drogas, a descriminalização do uso de drogas e a legalização da maconha a curto prazo. Propõe adotar as 16 medidas contra o encarceramento em massa do IBCCRIM, cotas raciais nas forças de segurança e fim da privatização dos presídios. Também prevê ocupação de territórios dominados pelo crime organizado com serviços públicos e a expropriação do sistema financeiro que financia o crime organizado.</t>
+          <t>O plano propõe uma política de segurança dos direitos no lugar da atual segurança pública, com desmilitarização completa, unificação das polícias e ciclo completo de formação. Defende o fim da política de guerra às drogas, a descriminalização do uso de drogas e a legalização da maconha a curto prazo. Propõe adotar um conjunto de medidas técnicas, formuladas por especialistas em ciências criminais, para reduzir o encarceramento em massa, além de cotas raciais nas forças de segurança e fim da privatização dos presídios. Também prevê ocupação de territórios dominados pelo crime organizado com serviços públicos e a expropriação do sistema financeiro que financia o crime organizado.</t>
         </is>
       </c>
       <c r="F41" s="4" t="inlineStr">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>O programa propõe reconstrução radical do sistema político, com Orçamento Popular 100% deliberativo, convocação de uma Assembleia Constituinte de Novo Tipo e extinção do Senado, substituído por um Parlamento Unicameral. Defende a criação de Conselhos Populares em locais de trabalho, moradia e estudo, além da possibilidade de revogação de mandatos por meio de referendos populares. Propõe democratizar o Judiciário, com mandatos fixos de dez anos para tribunais superiores sob controle social, e democratizar os meios de comunicação, com fim dos monopólios privados e fortalecimento da EBC. Também prevê convocação imediata de concursados aprovados e ampliação de concursos públicos.</t>
+          <t>O programa propõe reconstrução radical do sistema político, com Orçamento Popular 100% deliberativo, convocação de uma nova Assembleia Constituinte com ampla participação popular, e extinção do Senado, substituído por um Parlamento Unicameral. Defende a criação de Conselhos Populares em locais de trabalho, moradia e estudo, além da possibilidade de revogação de mandatos por meio de referendos populares. Propõe democratizar o Judiciário, com mandatos fixos de dez anos para tribunais superiores sob controle social, e democratizar os meios de comunicação, com fim dos monopólios privados e fortalecimento da EBC. Também prevê convocação imediata de concursados aprovados e ampliação de concursos públicos.</t>
         </is>
       </c>
       <c r="F48" s="4" t="inlineStr">
@@ -2043,7 +2043,7 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>O plano prioriza a alfabetização pelo método fônico e cria o Programa Acolher, em que alunos com bom desempenho recebem remuneração para dar reforço aos colegas. Propõe gestão escolar baseada em resultados, financiamento vinculado a metas de aprendizagem e qualificação de professores por evidências científicas, além de escolas cívico-militares e escola em tempo integral. Defende educação livre de doutrinação político-partidária, respeitando os valores das famílias. No ensino técnico e superior, propõe parcerias com o setor produtivo, transferência da governança do ensino superior ao Ministério da Ciência, Tecnologia e Inovações, e um novo modelo de financiamento estudantil com pagamento proporcional à renda após o emprego. Também prevê voucher educacional quando faltar vaga na rede pública e ampliação de creches via voucher-creche.</t>
+          <t>O plano prioriza a alfabetização pelo método fônico e cria um programa em que alunos com bom desempenho recebem remuneração para dar reforço aos colegas. Propõe gestão escolar baseada em resultados, financiamento vinculado a metas de aprendizagem e qualificação de professores por evidências científicas, além de escolas cívico-militares e escola em tempo integral. Defende educação livre de doutrinação político-partidária, respeitando os valores das famílias. No ensino técnico e superior, propõe parcerias com o setor produtivo, transferência da governança do ensino superior ao Ministério da Ciência, Tecnologia e Inovações, e um novo modelo de financiamento estudantil com pagamento proporcional à renda após o emprego. Também prevê voucher educacional quando faltar vaga na rede pública e ampliação de creches via voucher-creche.</t>
         </is>
       </c>
       <c r="F50" s="4" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>O plano defende revisão da reforma tributária para reduzir o IVA e eliminar distorções, corte de ao menos 10 ministérios, redução de despesas e combate a supersalários, além de equilíbrio fiscal com regras claras de controle de gastos para reduzir a dívida pública, os juros e a inflação. Propõe simplificação da conta de luz, redução de impostos sobre energia, combustíveis e consumo, e crédito mais barato para famílias e empresas. Defende profissionalização das estatais e das agências reguladoras, combate à corrupção e maior transparência no uso de recursos públicos. Também prevê ampliação do crédito via CAIXA como "Banco da Prosperidade" e o programa Ganha-Ganha para dar histórico financeiro positivo a quem hoje é invisível ao sistema.</t>
+          <t>O plano defende revisão da reforma tributária para reduzir o IVA e eliminar distorções, corte de ao menos 10 ministérios, redução de despesas e combate a supersalários, além de equilíbrio fiscal com regras claras de controle de gastos para reduzir a dívida pública, os juros e a inflação. Propõe simplificação da conta de luz, redução de impostos sobre energia, combustíveis e consumo, e crédito mais barato para famílias e empresas. Defende profissionalização das estatais e das agências reguladoras, combate à corrupção e maior transparência no uso de recursos públicos. Também prevê ampliar o crédito por meio da CAIXA, dando histórico financeiro positivo a quem hoje é invisível ao sistema.</t>
         </is>
       </c>
       <c r="F51" s="4" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>Propõe prontuário eletrônico único integrado ao CPF e ao Gov.br, digitalização total do SUS com agendamento de consultas e exames por inteligência artificial, e correção da tabela SUS para remunerar melhor hospitais e clínicas. Prevê ampliação da Estratégia Saúde da Família, do Programa de Atendimento aos Idosos, de exames preventivos e da telessaúde, além de contratação de horários ociosos da rede privada para reduzir filas. Cria a Saúde para Elas, com unidades móveis, atenção à mulher e prevenção de câncer, e amplia o cuidado em saúde mental, incluindo TDAH, depressão, ansiedade e Alzheimer. Também prevê entrega domiciliar de remédios para idosos, pessoas com deficiência e doentes crônicos.</t>
+          <t>Propõe prontuário eletrônico único integrado ao CPF e ao Gov.br, digitalização total do SUS com agendamento de consultas e exames por inteligência artificial, e correção da tabela SUS para remunerar melhor hospitais e clínicas. Prevê ampliação da Estratégia Saúde da Família, do atendimento aos idosos, de exames preventivos e da telessaúde, além de contratação de horários ociosos da rede privada para reduzir filas. Cria um programa de atenção à saúde da mulher, com unidades móveis, prevenção de câncer e atendimento humanizado, e amplia o cuidado em saúde mental, incluindo TDAH, depressão, ansiedade e Alzheimer. Também prevê entrega domiciliar de remédios para idosos, pessoas com deficiência e doentes crônicos.</t>
         </is>
       </c>
       <c r="F52" s="4" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe tratar facções como organizações narcoterroristas, reduzir a maioridade penal de 18 para 16 anos e punir maiores de 14 anos por crimes graves. Prevê construção de novos presídios de segurança máxima (Complexo TREVA), fim da progressão de regime para crimes hediondos e castração química para estupradores e abusadores de crianças condenados. Propõe monitoramento por tornozeleira eletrônica de agressores de mulheres, um sistema nacional de reconhecimento facial (Muralha Brasileira) com mais de 1 milhão de novas câmeras, e dobrar os investimentos federais em segurança pública. Também cria o Sistema Nacional de Fronteira com tropas de elite e prevê penas mais duras para roubo e receptação de celulares.</t>
+          <t>O plano propõe tratar facções como organizações narcoterroristas, reduzir a maioridade penal de 18 para 16 anos e punir maiores de 14 anos por crimes graves. Prevê construção de novos presídios de segurança máxima, fim da progressão de regime para crimes hediondos e castração química para estupradores e abusadores de crianças condenados. Propõe monitoramento por tornozeleira eletrônica de agressores de mulheres, um sistema nacional de reconhecimento facial com mais de 1 milhão de novas câmeras, e dobrar os investimentos federais em segurança pública. Também cria uma força federal de fronteira com tropas de elite e prevê penas mais duras para roubo e receptação de celulares.</t>
         </is>
       </c>
       <c r="F53" s="4" t="inlineStr">
@@ -2148,7 +2148,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="105" customHeight="1">
+    <row r="54" ht="120" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>22</t>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>O plano prevê investimento de R$ 900 bilhões em quatro anos em rodovias, ferrovias, hidrovias, portos e aeroportos, com criação de Corredores Logísticos Inteligentes para reduzir o custo logístico. Propõe destravar a Ferrogrão, o trem de cargas ligando Mato Grosso ao Paraná e Santa Catarina, o Trem do Nordeste e a conclusão da Transnordestina. Defende financiamento público prioritário para metrô, trens e ônibus elétricos ou a biocombustível nas cidades, reduzindo o tempo de deslocamento urbano. Também prevê modernização dos marcos regulatórios e segurança jurídica para atrair investimento privado em infraestrutura.</t>
+          <t>O plano prevê investimento de R$ 900 bilhões em quatro anos em rodovias, ferrovias, hidrovias, portos e aeroportos, com criação de corredores logísticos inteligentes para reduzir o custo logístico. Propõe destravar a construção de uma ferrovia de cargas ligando o Mato Grosso ao Paraná e a Santa Catarina, um novo trem de passageiros no Nordeste e a conclusão de obras ferroviárias estruturantes na região. Defende financiamento público prioritário para metrô, trens e ônibus elétricos ou a biocombustível nas cidades, reduzindo o tempo de deslocamento urbano. Também prevê modernização dos marcos regulatórios e segurança jurídica para atrair investimento privado em infraestrutura.</t>
         </is>
       </c>
       <c r="F54" s="4" t="inlineStr">
@@ -2203,7 +2203,7 @@
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>O plano trata o meio ambiente como ativo estratégico, propondo licenciamento ambiental ágil com prazos definidos, meta de zerar o desmatamento ilegal até 2029 e combate a queimadas e crimes ambientais com uso de inteligência artificial e monitoramento por satélite. Defende ampliação do pagamento por serviços ambientais para quem preserva vegetação nativa, consolidação do mercado regulado de carbono e impulso à bioeconomia na Amazônia. Propõe fortalecer a fiscalização ambiental na Amazônia sem criminalizar ribeirinhos, extrativistas e pequenos produtores, e exigir transparência de ONGs financiadas do exterior. Também dá continuidade à universalização do saneamento básico via Marco Legal do Saneamento.</t>
+          <t>O plano trata o meio ambiente como ativo estratégico, propondo licenciamento ambiental ágil com prazos definidos, meta de zerar o desmatamento ilegal até 2029 e combate a queimadas e crimes ambientais com uso de inteligência artificial e monitoramento por satélite. Defende ampliação do pagamento por serviços ambientais para quem preserva vegetação nativa, consolidação do mercado regulado de carbono e impulso à bioeconomia na Amazônia. Propõe fortalecer a fiscalização ambiental na Amazônia sem criminalizar ribeirinhos, extrativistas e pequenos produtores, e exigir transparência de ONGs financiadas do exterior. Também dá continuidade à universalização do saneamento básico dentro do marco regulatório vigente.</t>
         </is>
       </c>
       <c r="F55" s="4" t="inlineStr">
@@ -2235,12 +2235,12 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>O plano mantém os programas sociais existentes e promete corrigir distorções e combater fraudes, tratando o benefício como ponto de partida para qualificação, emprego e crédito, não como destino permanente. Cria o Brasil por Elas, com Central da Mulher, aplicativo com assistente virtual ClarIA, bônus de internet, orientação financeira e o programa Ganha-Ganha para mulheres empreendedoras. Propõe ampliação de creches com voucher-creche, criação da Rede Nacional de Cuidado para idosos e pessoas com deficiência, e ampliação de instituições de longa permanência. Também prevê prioridade a beneficiários de programas sociais em qualificação profissional e retorno sem fila ao benefício após tentativa de emprego.</t>
+          <t>O plano mantém os programas sociais existentes e promete corrigir distorções e combater fraudes, tratando o benefício como ponto de partida para qualificação, emprego e crédito, não como destino permanente. Cria uma rede de apoio à mulher, com central de atendimento, aplicativo com assistente virtual por inteligência artificial, bônus de internet, orientação financeira e crédito voltado a empreendedoras. Propõe ampliação de creches com voucher-creche, criação de uma rede nacional de cuidado para idosos e pessoas com deficiência, e ampliação de instituições de longa permanência. Também prevê prioridade a beneficiários de programas sociais em qualificação profissional e retorno sem fila ao benefício após tentativa de emprego.</t>
         </is>
       </c>
       <c r="F56" s="4" t="inlineStr">
         <is>
-          <t>Programas sociais mantidos e usados como trampolim: creche, cuidado a idosos, Brasil por Elas e qualificação para sair da pobreza.</t>
+          <t>Programas sociais mantidos e usados como trampolim: creche, cuidado a idosos, apoio à mulher e qualificação para sair da pobreza.</t>
         </is>
       </c>
     </row>
@@ -2299,12 +2299,12 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe uma Estratégia Nacional de Inteligência Artificial para difundir IA entre micro, pequenas e médias empresas, priorizando indústria, agronegócio, saúde e logística. Defende o Brasil como produtor de tecnologia, aproveitando energia limpa, minerais críticos e talento nacional, com legislação de liberdade de criar e inovar, fortalecimento de parques tecnológicos, incubadoras e startups. Propõe unificar ciência e ensino superior sob o Ministério da Ciência, Tecnologia e Inovações, priorizando impacto produtivo e transferência de tecnologia das universidades à indústria. Também prevê fortalecimento da defesa cibernética e proteção de dados dos cidadãos.</t>
+          <t>O plano propõe uma estratégia nacional de inteligência artificial para difundir IA entre micro, pequenas e médias empresas, priorizando indústria, agronegócio, saúde e logística. Defende o Brasil como produtor de tecnologia, aproveitando energia limpa, minerais críticos e talento nacional, com legislação de liberdade de criar e inovar, fortalecimento de parques tecnológicos, incubadoras e startups. Propõe unificar ciência e ensino superior sob o Ministério da Ciência, Tecnologia e Inovações, priorizando impacto produtivo e transferência de tecnologia das universidades à indústria. Também prevê fortalecimento da defesa cibernética e proteção de dados dos cidadãos.</t>
         </is>
       </c>
       <c r="F58" s="4" t="inlineStr">
         <is>
-          <t>Estratégia Nacional de IA para pequenas empresas, mais patentes de tecnologia brasileira e proteção de dados dos cidadãos.</t>
+          <t>Estratégia nacional de IA para pequenas empresas, mais patentes de tecnologia brasileira e proteção de dados dos cidadãos.</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe reduzir gradualmente o custo do trabalho sem retirar direitos, criando contratos com menor custo para jovens de 18 a 24 anos no primeiro emprego e para desempregados com 50 anos ou mais. Defende o negociado sobre o legislado, jornada flexível e um banco nacional de vagas conectado ao RH das empresas. Propõe digitalizar e profissionalizar a gestão do INSS para acabar com a fila de mais de 3 milhões de requerimentos, e reeditar um pacote antifraude na Previdência para proteger aposentados de descontos indevidos. Também se posiciona contra a "República Sindical" e defende a manutenção do trabalho por aplicativos.</t>
+          <t>O plano propõe reduzir gradualmente o custo do trabalho sem retirar direitos, criando contratos com menor custo para jovens de 18 a 24 anos no primeiro emprego e para desempregados com 50 anos ou mais. Defende o negociado sobre o legislado, jornada flexível e um banco nacional de vagas conectado ao RH das empresas. Propõe digitalizar e profissionalizar a gestão do INSS para acabar com a fila de mais de 3 milhões de requerimentos, e reeditar um pacote antifraude na Previdência para proteger aposentados de descontos indevidos. Também se posiciona contra o modelo de sindicalismo obrigatório e defende a manutenção do trabalho por aplicativos.</t>
         </is>
       </c>
       <c r="F59" s="4" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe um "Tesouraço": corte de ao menos 10 ministérios, redução de cargos comissionados, combate a penduricalhos e supersalários, e ampla revisão de normas que travam a economia. Defende profissionalização das estatais e agências reguladoras, blindagem dos fundos de pensão contra indicação política e retomada do Programa Nacional de Desestatização. Propõe digitalizar 100% dos serviços públicos federais, com identidade digital única e assistentes de inteligência artificial que antecipam as necessidades do cidadão. Também prevê mais transparência e rastreabilidade das emendas parlamentares e reforma do pacto federativo para dar mais autonomia a estados e municípios.</t>
+          <t>O plano propõe um amplo programa de corte de gastos: eliminação de ao menos 10 ministérios, redução de cargos comissionados, combate a penduricalhos e supersalários, e ampla revisão de normas que travam a economia. Defende profissionalização das estatais e agências reguladoras, blindagem dos fundos de pensão contra indicação política e retomada do processo de privatização de estatais. Propõe digitalizar 100% dos serviços públicos federais, com identidade digital única e assistentes de inteligência artificial que antecipam as necessidades do cidadão. Também prevê mais transparência e rastreabilidade das emendas parlamentares e reforma do pacto federativo para dar mais autonomia a estados e municípios.</t>
         </is>
       </c>
       <c r="F60" s="4" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>O plano defende ampliação do Seguro Rural, da capacidade de armazenamento de safras e da titulação de pequenos proprietários rurais, retomando o ritmo alcançado no governo Bolsonaro. Propõe simplificar outorgas de irrigação, hoje com prazo médio de 24 meses, ampliar a área irrigada no Matopiba e no semiárido nordestino, e apoiar a produção nacional de fertilizantes a partir de potássio e fosfato. Defende segurança jurídica sólida sobre a propriedade rural, rastreabilidade completa das cadeias produtivas e autonomia para povos indígenas e quilombolas decidirem sobre atividades produtivas em suas terras. Também prevê criação de Corredores Logísticos Inteligentes para reduzir o custo de transporte da produção agrícola.</t>
+          <t>O plano defende ampliação do Seguro Rural, da capacidade de armazenamento de safras e da titulação de pequenos proprietários rurais, buscando recuperar o ritmo alcançado em gestões anteriores. Propõe simplificar outorgas de irrigação, hoje com prazo médio de 24 meses, ampliar a área irrigada no Matopiba e no semiárido nordestino, e apoiar a produção nacional de fertilizantes a partir de potássio e fosfato. Defende segurança jurídica sólida sobre a propriedade rural, rastreabilidade completa das cadeias produtivas e autonomia para povos indígenas e quilombolas decidirem sobre atividades produtivas em suas terras. Também prevê criação de corredores logísticos inteligentes para reduzir o custo de transporte da produção agrícola.</t>
         </is>
       </c>
       <c r="F61" s="4" t="inlineStr">
@@ -2404,7 +2404,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="120" customHeight="1">
+    <row r="62" ht="105" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
           <t>28</t>
@@ -2415,7 +2415,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
           <t>Educação</t>
@@ -2423,12 +2427,12 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>O plano de governo propõe garantir a alfabetização plena até o 2º ano e ampliar bolsas de estudo para engenharia, ciências, matemática e TIC. Destaca a valorização dos professores em salário, segurança e capacitação, além de programas como o Alphabyte, para ensino de computação e IA nas escolas, e o ForSuper, voltado a alunos superdotados. Prevê ainda o Crédito Mirim, que bonifica estudantes da rede pública, e a Alfabetização Precoce, para estimular o desenvolvimento cognitivo infantil. A Universidade Federal Digital (UFD) e o programa GVE (Graduação, Virtualização e Empresarização) buscam ampliar o acesso ao ensino superior digital e conectar empresas e universidades.</t>
+          <t>O plano de governo propõe garantir a alfabetização plena até o 2º ano e ampliar bolsas de estudo para engenharia, ciências, matemática e TIC. Destaca a valorização dos professores em salário, segurança e capacitação, além de programas de ensino de computação e IA nas escolas e de atendimento especializado a alunos superdotados. Prevê ainda bonificação para estudantes de destaque da rede pública e ações de estímulo ao desenvolvimento cognitivo infantil desde a primeira infância. Propõe a criação de uma universidade federal digital, com graduação online que conecta empresas e universidades, ampliando o acesso ao ensino superior.</t>
         </is>
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>Alfabetização plena até o 2º ano, valorização de professores, ensino de IA e Universidade Federal Digital para todos.</t>
+          <t>Alfabetização plena até o 2º ano, valorização de professores, ensino de IA e universidade federal digital para todos.</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2447,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C63" s="3" t="inlineStr"/>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
           <t>Economia</t>
@@ -2451,12 +2459,12 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>A proposta central é transformar o empreendedorismo em política nacional de desenvolvimento, com a criação do Ministério da Empresarização e regime tributário simplificado para microempreendedores. Prevê abertura automática de empresas pelo CPF Digital em 24h, um Marco Nacional das Empresas Inovadoras para startups e o Renegocia Brasil, programa de renegociação de dívidas de brasileiros negativados. Também propõe redução progressiva da carga tributária, reforma tributária simplificada, câmbio flutuante e metas para conter a inflação como tripé econômico. O plano defende responsabilidade fiscal, com redução gradual da dívida/PIB e fim de subsídios sem retorno comprovado, mantendo o salário mínimo como o melhor da América do Sul.</t>
+          <t>A proposta central é transformar o empreendedorismo em política nacional de desenvolvimento, com a criação de um ministério dedicado ao tema e regime tributário simplificado para microempreendedores. Prevê abertura automática de empresas em até 24h por meio de identificação digital unificada, um novo marco legal para empresas inovadoras (startups) e um programa de renegociação de dívidas para brasileiros negativados. Também propõe redução progressiva da carga tributária, reforma tributária simplificada, câmbio flutuante e metas para conter a inflação como tripé econômico. O plano defende responsabilidade fiscal, com redução gradual da dívida/PIB e fim de subsídios sem retorno comprovado, mantendo o salário mínimo como o melhor da América do Sul.</t>
         </is>
       </c>
       <c r="F63" s="4" t="inlineStr">
         <is>
-          <t>Empresarização como política nacional: menos burocracia, mais crédito, reforma tributária, responsabilidade fiscal e redução de impostos.</t>
+          <t>Empreendedorismo como política nacional: menos burocracia, mais crédito, reforma tributária, responsabilidade fiscal.</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2479,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C64" s="3" t="inlineStr"/>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Saúde</t>
@@ -2479,7 +2491,7 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>O plano prevê reduzir filas e ampliar o acesso à atenção básica, com prontuário único nacional e telemedicina integrada ao SUS. Propõe o lançamento do Programa Nacional de Saúde Mental e de ações de prevenção de doenças por meio do incentivo a hábitos saudáveis. O Pró-Saúde busca dar mais eficiência à rede pública e atendimento mais respeitoso aos usuários, enquanto os Polos Tecnológicos de Saúde (PTS) pretendem criar infraestrutura tecnológica para o atendimento. Também há previsão de uso de inteligência artificial aplicada ao SUS.</t>
+          <t>O plano prevê reduzir filas e ampliar o acesso à atenção básica, com prontuário único nacional e telemedicina integrada ao SUS. Propõe o lançamento de um programa nacional de saúde mental e de ações de prevenção de doenças por meio do incentivo a hábitos saudáveis. Busca dar mais eficiência à rede pública e atendimento mais respeitoso aos usuários, com a criação de polos tecnológicos de saúde para ampliar a infraestrutura de atendimento. Também há previsão de uso de inteligência artificial aplicada ao SUS.</t>
         </is>
       </c>
       <c r="F64" s="4" t="inlineStr">
@@ -2499,7 +2511,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr"/>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
           <t>Segurança</t>
@@ -2507,7 +2523,7 @@
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe um Plano Nacional de Combate às Facções, com integração de inteligência financeira e confisco ampliado de patrimônio de criminosos. Prevê modernização das leis penais contra organizações criminosas, sistema integrado de vigilância nas fronteiras com drones e satélites, e uma Rede Nacional de Proteção para defesa da mulher. O sistema prisional seria transformado em centros de ressocialização, com trabalho remunerado e ensino técnico obrigatório, além de um programa específico contra dependência química. Também prevê combate à corrupção com transparência total dos gastos públicos e uso de IA para identificar fraudes, além de um programa nacional contra furto e roubo de veículos e celulares.</t>
+          <t>O plano propõe um plano nacional de combate às facções criminosas, com integração de inteligência financeira e confisco ampliado de patrimônio de criminosos. Prevê modernização das leis penais contra organizações criminosas, sistema integrado de vigilância nas fronteiras com drones e satélites, e uma rede nacional de proteção para defesa da mulher. O sistema prisional seria transformado em centros de ressocialização, com trabalho remunerado e ensino técnico obrigatório, além de um programa específico contra dependência química. Também prevê combate à corrupção com transparência total dos gastos públicos e uso de IA para identificar fraudes, além de um programa nacional contra furto e roubo de veículos e celulares.</t>
         </is>
       </c>
       <c r="F65" s="4" t="inlineStr">
@@ -2527,7 +2543,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr"/>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Transporte</t>
@@ -2535,12 +2555,12 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>O plano prevê um Plano Nacional de Infraestrutura Integrada, com modernização do modelo de concessões e conclusão de mais de 20 mil obras públicas federais inacabadas. Propõe a integração ferroviária nacional, incluindo o corredor Norte-Sul completo e a integração ferroviária agroindustrial, além da concessão e duplicação de rodovias estratégicas. Contempla ainda ampliação da conectividade regional em aeroportos, modernização dos corredores de exportação portuários com janela única portuária, e o Programa Brasil Mobilidade 2035 para o setor automotivo.</t>
+          <t>O plano prevê um plano nacional de infraestrutura integrada, com modernização do modelo de concessões e conclusão de mais de 20 mil obras públicas federais inacabadas. Propõe a integração ferroviária nacional, incluindo o corredor Norte-Sul completo e a integração ferroviária agroindustrial, além da concessão e duplicação de rodovias estratégicas. Contempla ainda ampliação da conectividade regional em aeroportos, modernização dos corredores de exportação portuários com janela única portuária, e um programa de incentivo ao setor automotivo com metas até 2035.</t>
         </is>
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>Integração ferroviária, rodovias duplicadas, aeroportos conectados, portos modernizados e Programa Brasil Mobilidade 2035.</t>
+          <t>Integração ferroviária, rodovias duplicadas, aeroportos conectados, portos modernizados e plano para o setor automotivo.</t>
         </is>
       </c>
     </row>
@@ -2555,7 +2575,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr"/>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
           <t>Meio Ambiente</t>
@@ -2563,7 +2587,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>O plano prevê lançar o Programa Nacional de Bioeconomia para geração de renda e um programa de recuperação de áreas degradadas e recomposição de nascentes estratégicas para segurança hídrica. Propõe regulamentar e consolidar o mercado brasileiro de carbono, atraindo investimentos privados para conservação ambiental, além de combater o desmatamento ilegal. Também prevê uma política que remunere serviços ambientais prestados por florestas em pé e ações de combate ao comércio ilegal e proteção aos direitos dos animais.</t>
+          <t>O plano prevê lançar um programa nacional de bioeconomia para geração de renda e um programa de recuperação de áreas degradadas e recomposição de nascentes estratégicas para segurança hídrica. Propõe regulamentar e consolidar o mercado brasileiro de carbono, atraindo investimentos privados para conservação ambiental, além de combater o desmatamento ilegal. Também prevê uma política que remunere serviços ambientais prestados por florestas em pé e ações de combate ao comércio ilegal e proteção aos direitos dos animais.</t>
         </is>
       </c>
       <c r="F67" s="4" t="inlineStr">
@@ -2583,7 +2607,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr"/>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
           <t>Desenvolvimento Social</t>
@@ -2591,12 +2619,12 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>O plano mantém o Programa Bolsa Família e assegura respeito aos direitos constitucionais de povos indígenas, quilombolas e povos tradicionais, com regularização fundiária e programas de bioeconomia para essas comunidades. Prevê a universalização de creches para famílias vulneráveis, monitoramento nacional do desenvolvimento infantil e o Programa Nacional de Fortalecimento da Família, além de ações de combate à violência doméstica e paternidade responsável. Defende o combate à pobreza por meio da emancipação econômica, com promoção de acessibilidade e inclusão para pessoas com deficiência, em vez da dependência permanente de programas assistenciais. Também propõe o Programa de Liberdade para Adquirir Residência (LAR), para corrigir imperfeições dos programas habitacionais.</t>
+          <t>O plano mantém o programa de transferência de renda para famílias em situação de vulnerabilidade e assegura respeito aos direitos constitucionais de povos indígenas, quilombolas e povos tradicionais, com regularização fundiária e programas de bioeconomia para essas comunidades. Prevê a universalização de creches para famílias vulneráveis, monitoramento nacional do desenvolvimento infantil e um programa nacional de fortalecimento da família, além de ações de combate à violência doméstica e paternidade responsável. Defende o combate à pobreza por meio da emancipação econômica, com promoção de acessibilidade e inclusão para pessoas com deficiência, em vez da dependência permanente de programas assistenciais. Também propõe um novo programa habitacional para corrigir imperfeições dos programas já existentes.</t>
         </is>
       </c>
       <c r="F68" s="4" t="inlineStr">
         <is>
-          <t>Bolsa Família mantido, apoio a povos tradicionais e pessoas com deficiência, e combate à pobreza pela emancipação econômica.</t>
+          <t>Transferência de renda mantida, apoio a povos tradicionais e pessoas com deficiência, combate à pobreza pela emancipação.</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2639,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C69" s="3" t="inlineStr"/>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
           <t>Relações Internacionais</t>
@@ -2619,7 +2651,7 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>O plano busca dobrar as exportações brasileiras e o fluxo comercial com a América Latina, além de destravar o potencial do acordo Mercosul-União Europeia. Prevê retomada do convívio diplomático com os Estados Unidos, com cooperação em IA, semicondutores e minerais raros, e uma estratégia própria para relações com a Ásia, incluindo Brasil-Índia, ASEAN e atualização do modelo de relacionamento com a China. Propõe também um novo eixo geopolítico Sul-Sul e um modelo estratégico de integração com a África, além de ampliar a atuação da APEX Brasil na promoção de exportações e investimentos.</t>
+          <t>O plano busca dobrar as exportações brasileiras e o fluxo comercial com a América Latina, além de destravar o potencial do acordo comercial entre o Mercosul e a União Europeia. Prevê retomada do convívio diplomático com os Estados Unidos, com cooperação em IA, semicondutores e minerais raros, e uma estratégia própria para relações com a Ásia, incluindo laços mais estreitos com a Índia, o bloco ASEAN e atualização do modelo de relacionamento com a China. Propõe também um novo eixo geopolítico Sul-Sul e um modelo estratégico de integração com a África, além de ampliar a atuação da agência nacional de promoção de exportações e investimentos.</t>
         </is>
       </c>
       <c r="F69" s="4" t="inlineStr">
@@ -2639,7 +2671,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C70" s="3" t="inlineStr"/>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
           <t>Ciência e Tecnologia</t>
@@ -2647,16 +2683,16 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>O plano prevê lançar uma Estratégia Nacional de Inteligência Artificial, com um Laboratório Nacional de IA e aplicações de IA na saúde (SUS) e na educação pública. Propõe universalizar internet de alta velocidade e cobertura 5G em todos os municípios, além de levar internet a 100% das escolas públicas por meio do Programa Amazônia Conectada. Contempla ainda a criação da Universidade Federal Digital, com graduação tecnológica online e certificações profissionais rápidas, um Comando Nacional de Defesa Digital para cibersegurança, e incentivos para datacenters e para um polo nacional de produção de jogos digitais (Tech Gamer).</t>
+          <t>O plano prevê lançar uma estratégia nacional de inteligência artificial, com um laboratório nacional de pesquisa em IA e aplicações de IA na saúde (SUS) e na educação pública. Propõe universalizar internet de alta velocidade e cobertura 5G em todos os municípios, além de levar internet a 100% das escolas públicas por meio de um programa de conectividade voltado a regiões remotas. Contempla ainda a criação de uma universidade federal digital, com graduação tecnológica online e certificações profissionais rápidas, um órgão nacional de defesa cibernética, e incentivos para datacenters e para um polo nacional de produção de jogos digitais.</t>
         </is>
       </c>
       <c r="F70" s="4" t="inlineStr">
         <is>
-          <t>Estratégia Nacional de IA, 5G em todos municípios, Universidade Federal Digital e cibersegurança nacional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="90" customHeight="1">
+          <t>Estratégia de IA, 5G em todos municípios, universidade federal digital e defesa cibernética nacional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="105" customHeight="1">
       <c r="A71" s="2" t="inlineStr">
         <is>
           <t>28</t>
@@ -2667,7 +2703,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr"/>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
           <t>Trabalho e Previdência</t>
@@ -2675,16 +2715,16 @@
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>O plano garante a manutenção do valor do salário mínimo como o melhor da América do Sul, valorizando o trabalhador brasileiro. Prevê a reorientação da formação profissional do Sistema S para a indústria do futuro e o lançamento do Programa V.E.T. (Vocação, Educação e Treinamento), com mapeamento técnico de talentos para direcionar o capital humano. No sistema prisional, prevê trabalho remunerado e ensino técnico obrigatório como parte da ressocialização. O documento não apresenta propostas específicas sobre reforma da previdência.</t>
+          <t>O plano garante a manutenção do valor do salário mínimo como o melhor da América do Sul, valorizando o trabalhador brasileiro. Prevê a reorientação da formação profissional oferecida pelo sistema de aprendizagem industrial para a indústria do futuro e o lançamento de um programa de mapeamento técnico de talentos, com foco em vocação, educação e treinamento, para direcionar o capital humano. No sistema prisional, prevê trabalho remunerado e ensino técnico obrigatório como parte da ressocialização. O documento não apresenta propostas específicas sobre reforma da previdência.</t>
         </is>
       </c>
       <c r="F71" s="4" t="inlineStr">
         <is>
-          <t>Salário mínimo o melhor da América do Sul, reorientação do Sistema S e Programa V.E.T. de formação profissional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="105" customHeight="1">
+          <t>Salário mínimo o melhor da América do Sul, reorientação da formação profissional e mapeamento de talentos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="120" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
           <t>28</t>
@@ -2695,7 +2735,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C72" s="3" t="inlineStr"/>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
           <t>Gestão Pública</t>
@@ -2703,12 +2747,12 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe um Estado enxuto, eficiente, digital e focado em resultados, com digitalização de 100% dos serviços federais e implantação de gestão por resultados com painéis de KPIs em todos os órgãos. Prevê desburocratização com mutirão de revogação de normas obsoletas e a regra 'one in, one out', além do Programa de Desestatização Prioritária e profissionalização da gestão das estatais. Propõe o Governo Itinerante, levando presidente e ministros a todas as regiões do país, um marketplace nacional de compras governamentais com IA contra fraudes em licitações, e a reforma tributária com simplificação do modelo e redução da carga tributária.</t>
+          <t>O plano propõe um Estado enxuto, eficiente, digital e focado em resultados, com digitalização de 100% dos serviços federais e implantação de gestão por resultados com painéis de indicadores em todos os órgãos. Prevê desburocratização com mutirão de revogação de normas obsoletas e a regra 'one in, one out', além de um programa de desestatização de empresas públicas prioritárias e profissionalização da gestão das estatais. Propõe levar o presidente e os ministros a todas as regiões do país por meio de um governo itinerante, um marketplace nacional de compras governamentais com IA contra fraudes em licitações, e a reforma tributária com simplificação do modelo e redução da carga tributária.</t>
         </is>
       </c>
       <c r="F72" s="4" t="inlineStr">
         <is>
-          <t>Estado digital e enxuto: desburocratização, desestatização, governo itinerante e reforma tributária simplificada.</t>
+          <t>Estado digital e enxuto: desburocratização, desestatização de estatais, governo itinerante e reforma tributária.</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2767,11 @@
           <t>Pablo Marçal</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr"/>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>União Brasil</t>
+        </is>
+      </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
           <t>Agricultura</t>
@@ -2731,7 +2779,7 @@
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>O plano busca a liderança global do Brasil em segurança alimentar e a integração do agronegócio à cadeia logística nacional. Propõe um Plano Nacional de Irrigação, seguro rural universal e expansão da armazenagem agrícola, além de desenvolvimento tecnológico das cadeias produtivas voltado a características regionais e aos micro e pequenos produtores rurais. Também prevê integração ferroviária agroindustrial e modernização dos corredores portuários de exportação para escoamento da produção.</t>
+          <t>O plano busca a liderança global do Brasil em segurança alimentar e a integração do agronegócio à cadeia logística nacional. Propõe um plano nacional de irrigação, seguro rural universal e expansão da armazenagem agrícola, além de desenvolvimento tecnológico das cadeias produtivas voltado a características regionais e aos micro e pequenos produtores rurais. Também prevê integração ferroviária agroindustrial e modernização dos corredores portuários de exportação para escoamento da produção.</t>
         </is>
       </c>
       <c r="F73" s="4" t="inlineStr">
@@ -2746,7 +2794,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B74" s="3" t="inlineStr"/>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2759,12 +2811,12 @@
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>O PCO defende ensino público, gratuito e de qualidade, com mais verbas exclusivamente para a rede pública e revogação das reformas educacionais dos últimos governos. Propõe fim dos vestibulares com livre ingresso nas universidades, estatização do ensino pago e piso salarial nacional de pelo menos R$8,5 mil para professores, com jornada máxima de 30 horas semanais. Defende a gestão das escolas e universidades pela própria comunidade escolar, com eleição direta de diretores e um governo tripartite de estudantes, professores e funcionários nas universidades. Também critica a proibição do uso de celulares nas escolas.</t>
+          <t>Defende ensino público, gratuito e de qualidade, com mais verbas exclusivamente para a rede pública e revogação das reformas educacionais dos últimos governos. Propõe fim dos vestibulares com livre ingresso nas universidades, estatização do ensino pago e piso salarial nacional de pelo menos R$8,5 mil para professores, com jornada máxima de 30 horas semanais. Defende a gestão das escolas e universidades pela própria comunidade escolar, com eleição direta de diretores e um governo tripartite de estudantes, professores e funcionários nas universidades. Também critica a proibição do uso de celulares nas escolas.</t>
         </is>
       </c>
       <c r="F74" s="4" t="inlineStr">
         <is>
-          <t>PCO quer educação pública, gratuita, sem vestibular, com gestão democrática das escolas e piso de R$8,5 mil para professores.</t>
+          <t>Quer educação pública, gratuita, sem vestibular, com gestão democrática das escolas e piso de R$8,5 mil para professores.</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2826,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr"/>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2787,12 +2843,12 @@
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>O PCO propõe cancelar todas as privatizações realizadas (Eletrobras, Vale, bancos, telefonia) e reestatizar essas empresas, com a Petrobras 100% estatal sob controle dos trabalhadores. Defende a nacionalização das reservas minerais e das terras raras, redução imediata de 50% no preço dos combustíveis e fim da paridade com o dólar. No sistema financeiro, propõe redução imediata dos juros, estatização dos bancos em um banco estatal único, fim da independência do Banco Central e cancelamento das dívidas externa e interna. Propõe ainda fim dos impostos sobre consumo e salários, com tributação apenas sobre lucros dos capitalistas e grandes fortunas.</t>
+          <t>Propõe cancelar todas as privatizações realizadas (Eletrobras, Vale, bancos, telefonia) e reestatizar essas empresas, com a Petrobras 100% estatal sob controle dos trabalhadores. Defende a nacionalização das reservas minerais e das terras raras, redução imediata de 50% no preço dos combustíveis e fim da paridade com o dólar. No sistema financeiro, propõe redução imediata dos juros, estatização dos bancos em um banco estatal único, fim da independência do Banco Central e cancelamento das dívidas externa e interna. Propõe ainda fim dos impostos sobre consumo e salários, com tributação apenas sobre lucros dos capitalistas e grandes fortunas.</t>
         </is>
       </c>
       <c r="F75" s="4" t="inlineStr">
         <is>
-          <t>PCO defende estatizar bancos e empresas privatizadas, cancelar dívida pública, reduzir juros e taxar só grandes fortunas.</t>
+          <t>Defende estatizar bancos e empresas privatizadas, cancelar dívida pública, reduzir juros e taxar só grandes fortunas.</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2858,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr"/>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2815,12 +2875,12 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>O PCO defende o fim da privatização da saúde e mais verbas para o SUS, sem limite de gastos para salvar vidas. Propõe um plano de emergência para construir hospitais e postos de saúde em todo o país, além de retomar o programa Mais Médicos e validar imediatamente diplomas de médicos brasileiros e estrangeiros. Defende a abertura de centenas de novos cursos de medicina e enfermagem, com livre acesso sem vestibular nas universidades públicas, para suprir a falta de profissionais. Propõe piso salarial de R$8 mil para os profissionais da saúde.</t>
+          <t>Defende o fim da privatização da saúde e mais verbas para o SUS, sem limite de gastos para salvar vidas. Propõe um plano de emergência para construir hospitais e postos de saúde em todo o país, além de retomar um programa de contratação emergencial de médicos e validar imediatamente diplomas de médicos brasileiros e estrangeiros. Defende a abertura de centenas de novos cursos de medicina e enfermagem, com livre acesso sem vestibular nas universidades públicas, para suprir a falta de profissionais. Propõe piso salarial de R$8 mil para os profissionais da saúde.</t>
         </is>
       </c>
       <c r="F76" s="4" t="inlineStr">
         <is>
-          <t>PCO quer mais verbas ao SUS, plano de emergência para hospitais, volta do Mais Médicos e piso de R$8 mil na saúde.</t>
+          <t>Quer mais verbas ao SUS, plano de emergência para hospitais, contratação emergencial de médicos e piso de R$8 mil na saúde.</t>
         </is>
       </c>
     </row>
@@ -2830,7 +2890,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B77" s="3" t="inlineStr"/>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2843,12 +2907,12 @@
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>O PCO denuncia a repressão policial, responsabilizando a polícia por milhares de mortes anuais, e propõe a dissolução da polícia militar e de todo o aparato repressivo do Estado. Defende o direito de autodefesa dos trabalhadores da cidade e do campo, com a formação de comitês de autodefesa nas comunidades urbanas, rurais e indígenas. O programa também associa a questão da segurança à liberdade de expressão, opondo-se à censura e defendendo o fim do controle da mídia por grandes famílias.</t>
+          <t>Denuncia a repressão policial, responsabilizando a polícia por milhares de mortes anuais, e propõe a dissolução da polícia militar e de todo o aparato repressivo do Estado. Defende o direito de autodefesa dos trabalhadores da cidade e do campo, com a formação de comitês de autodefesa nas comunidades urbanas, rurais e indígenas. Também associa a questão da segurança à liberdade de expressão, opondo-se à censura e defendendo o fim do controle da mídia por grandes famílias.</t>
         </is>
       </c>
       <c r="F77" s="4" t="inlineStr">
         <is>
-          <t>PCO propõe dissolver a polícia militar e criar comitês de autodefesa dos trabalhadores nas cidades e no campo.</t>
+          <t>Propõe dissolver a polícia militar e criar comitês de autodefesa dos trabalhadores nas cidades e no campo.</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2922,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr"/>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2871,12 +2939,12 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>O tema do transporte aparece de forma pontual no programa, associado à luta contra o desemprego. O PCO propõe passe livre nos transportes públicos para desempregados e trabalhadores da economia informal, como medida emergencial diante da crise de emprego. O documento não apresenta um plano amplo de mobilidade urbana ou de infraestrutura de transporte.</t>
+          <t>O tema do transporte aparece de forma pontual no programa, associado à luta contra o desemprego. Propõe passe livre nos transportes públicos para desempregados e trabalhadores da economia informal, como medida emergencial diante da crise de emprego. Não apresenta um plano amplo de mobilidade urbana ou de infraestrutura de transporte.</t>
         </is>
       </c>
       <c r="F78" s="4" t="inlineStr">
         <is>
-          <t>PCO propõe passe livre no transporte para desempregados e trabalhadores informais.</t>
+          <t>Defende passe livre no transporte para desempregados e trabalhadores informais.</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2954,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B79" s="3" t="inlineStr"/>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2906,7 +2978,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr"/>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2919,12 +2995,12 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>O PCO propõe um plano nacional de construção de milhões de moradias populares para garantir habitação digna à população, com expropriação de imóveis vagos de especuladores e proibição de despejos e desocupações. Defende ainda um auxílio emergencial efetivo e Bolsa Família de pelo menos um salário mínimo enquanto durar a crise social atual. O programa também pede mais verbas para os serviços públicos essenciais e o fim do teto de gastos que restringe investimentos sociais.</t>
+          <t>Propõe um plano nacional de construção de milhões de moradias populares para garantir habitação digna à população, com expropriação de imóveis vagos de especuladores e proibição de despejos e desocupações. Defende ainda um auxílio emergencial efetivo e um programa de transferência de renda de pelo menos um salário mínimo por família enquanto durar a crise social atual. Também pede mais verbas para os serviços públicos essenciais e o fim do teto de gastos que restringe investimentos sociais.</t>
         </is>
       </c>
       <c r="F80" s="4" t="inlineStr">
         <is>
-          <t>PCO quer moradia popular em massa, fim de despejos, Bolsa Família de um salário mínimo e fim do teto de gastos.</t>
+          <t>Propõe um plano de moradia popular em massa, fim de despejos, renda mínima de um salário mínimo por família e fim do teto de gastos.</t>
         </is>
       </c>
     </row>
@@ -2934,7 +3010,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B81" s="3" t="inlineStr"/>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2947,12 +3027,12 @@
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>O PCO se posiciona contra a internacionalização da Amazônia e qualquer ingerência estrangeira na região, defendendo a soberania nacional e o controle das riquezas amazônicas pelas organizações populares e indígenas. Manifesta apoio a Cuba, Nicarágua, Venezuela e à luta do povo boliviano, opondo-se à ingerência dos Estados Unidos e da OEA na América Latina. Declara ainda solidariedade aos povos que resistem ao imperialismo em conflitos internacionais, citando Palestina, Irã e Rússia.</t>
+          <t>Posiciona-se contra a internacionalização da Amazônia e qualquer ingerência estrangeira na região, defendendo a soberania nacional e o controle das riquezas amazônicas pelas organizações populares e indígenas. Manifesta apoio a Cuba, Nicarágua, Venezuela e à luta do povo boliviano, opondo-se à ingerência dos Estados Unidos e da OEA na América Latina. Declara ainda solidariedade aos povos que resistem ao imperialismo em conflitos internacionais, citando Palestina, Irã e Rússia.</t>
         </is>
       </c>
       <c r="F81" s="4" t="inlineStr">
         <is>
-          <t>PCO defende soberania na Amazônia, apoia Cuba, Venezuela, Nicarágua e é contra ingerência dos EUA na América Latina.</t>
+          <t>Defende soberania na Amazônia, apoia Cuba, Venezuela, Nicarágua e é contra ingerência dos EUA na América Latina.</t>
         </is>
       </c>
     </row>
@@ -2962,7 +3042,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr"/>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2982,7 +3066,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr"/>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -2995,12 +3083,12 @@
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>O PCO propõe reposição integral de 100% das perdas salariais, aumento emergencial de 50% dos salários e um salário mínimo vital de ao menos R$7.500. Defende a redução da jornada de trabalho para 35 horas semanais sem redução salarial, proibição de demissões e salário-desemprego igual ao último salário recebido. Propõe ainda a revogação completa da reforma trabalhista e da reforma da Previdência, com aposentadoria após 25 anos de trabalho para mulheres e 30 para homens, reajuste de 100% das perdas em aposentadorias e pensões, e fim dos privilégios previdenciários de militares e juízes.</t>
+          <t>Propõe reposição integral de 100% das perdas salariais, aumento emergencial de 50% dos salários e um salário mínimo vital de ao menos R$7.500. Defende a redução da jornada de trabalho para 35 horas semanais sem redução salarial, proibição de demissões e salário-desemprego igual ao último salário recebido. Propõe ainda a revogação completa da reforma trabalhista e da reforma da Previdência, com aposentadoria após 25 anos de trabalho para mulheres e 30 para homens, reajuste de 100% das perdas em aposentadorias e pensões, e fim dos privilégios previdenciários de militares e juízes.</t>
         </is>
       </c>
       <c r="F83" s="4" t="inlineStr">
         <is>
-          <t>PCO quer repor 100% das perdas salariais, jornada de 35h, fim da reforma trabalhista e da Previdência.</t>
+          <t>Quer repor 100% das perdas salariais, jornada de 35h, fim da reforma trabalhista e da Previdência.</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3098,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr"/>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -3023,12 +3115,12 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>O PCO defende o fim da terceirização no setor público, estabilidade para servidores contratados precariamente e a realização periódica de concursos públicos, além do fim do teto de gastos e da Lei de Responsabilidade Fiscal. O programa também propõe o fim do que chama de 'ditadura do Judiciário', incluindo a extinção do Supremo Tribunal Federal e a eleição popular de juízes e procuradores com mandatos revogáveis. Defende ainda liberdade total de organização partidária, com o fim de regras como a 'ficha limpa' e a 'cláusula de barreira'.</t>
+          <t>Defende o fim da terceirização no setor público, estabilidade para servidores contratados precariamente e a realização periódica de concursos públicos, além do fim do teto de gastos e da Lei de Responsabilidade Fiscal. Propõe ainda o fim do que chama de 'ditadura do Judiciário', incluindo a extinção do Supremo Tribunal Federal e a eleição popular de juízes e procuradores com mandatos revogáveis. Defende ainda liberdade total de organização partidária, com o fim de regras como a 'ficha limpa' e a 'cláusula de barreira'.</t>
         </is>
       </c>
       <c r="F84" s="4" t="inlineStr">
         <is>
-          <t>PCO quer fim do teto de gastos, concursos públicos periódicos e extinção do STF com eleição popular de juízes.</t>
+          <t>Busca fim do teto de gastos, concursos públicos periódicos e extinção do STF com eleição popular de juízes.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3130,11 @@
           <t>29</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr"/>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>Rui Costa</t>
+        </is>
+      </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
           <t>Partido da Causa Operária (PCO)</t>
@@ -3051,16 +3147,16 @@
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>O PCO propõe uma reforma agrária ampla, com expropriação dos latifúndios e assentamento imediato dos sem-terra acampados em todo o país. Defende a demarcação e posse das terras indígenas retomadas, com expulsão dos latifundiários que as invadiram, e a punição de responsáveis por assassinatos de trabalhadores e lideranças da luta pela terra. Propõe ainda o direito de autodefesa e armamento para trabalhadores do campo e povos indígenas, e a ocupação de latifúndios para garantir terra e produção de alimentos à classe trabalhadora.</t>
+          <t>Propõe uma reforma agrária ampla, com expropriação dos latifúndios e assentamento imediato dos sem-terra acampados em todo o país. Defende a demarcação e posse das terras indígenas retomadas, com expulsão dos latifundiários que as invadiram, e a punição de responsáveis por assassinatos de trabalhadores e lideranças da luta pela terra. Propõe ainda o direito de autodefesa e armamento para trabalhadores do campo e povos indígenas, e a ocupação de latifúndios para garantir terra e produção de alimentos à classe trabalhadora.</t>
         </is>
       </c>
       <c r="F85" s="4" t="inlineStr">
         <is>
-          <t>PCO propõe reforma agrária com expropriação de latifúndios e demarcação de terras indígenas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="90" customHeight="1">
+          <t>Prevê reforma agrária com expropriação de latifúndios e demarcação de terras indígenas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="105" customHeight="1">
       <c r="A86" s="2" t="inlineStr">
         <is>
           <t>30</t>
@@ -3083,7 +3179,7 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>O plano defende ampliar creches e pré-escolas com parcerias privadas, priorizando a aprendizagem e a alfabetização na idade certa. Propõe fortalecer o Saeb, modernizar a BNCC, valorizar professores por desempenho e profissionalizar a gestão escolar. No ensino médio, quer expandir a educação profissional e vincular o programa Pé-de-Meia ao desempenho dos alunos. Defende também mais liberdade às famílias, com escolas cívico-militares, conveniadas e regulamentação do homeschooling, além de reitores escolhidos por critérios técnicos nas universidades federais.</t>
+          <t>O plano defende ampliar creches e pré-escolas com parcerias privadas, priorizando a aprendizagem e a alfabetização na idade certa. Propõe fortalecer o Saeb, modernizar a BNCC, valorizar professores por desempenho e profissionalizar a gestão escolar. No ensino médio, quer expandir a educação profissional e vincular o programa de transferência de renda para estudantes do ensino médio ao desempenho dos alunos. Defende também mais liberdade às famílias, com escolas cívico-militares, conveniadas e regulamentação do homeschooling, além de reitores escolhidos por critérios técnicos nas universidades federais.</t>
         </is>
       </c>
       <c r="F86" s="4" t="inlineStr">
@@ -3211,7 +3307,7 @@
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe o maior portfólio de investimentos em infraestrutura da história do país, com forte participação do capital privado via concessões e PPPs. Defende reunificar o Ministério da Infraestrutura, modernizar a malha ferroviária com autorizações e concessões, expandir portos e aeroportos com mais participação privada e consolidar as hidrovias como corredor estratégico. Propõe também modernizar a gestão rodoviária com contratos de longo prazo e tecnologia de monitoramento, além de instituir uma política nacional de mobilidade urbana para expandir metrôs, trens e VLTs nas grandes regiões metropolitanas. Busca ainda simplificar o licenciamento ambiental e criar um regime de 'Projetos de Interesse Nacional' para acelerar obras estratégicas.</t>
+          <t>O plano propõe o maior portfólio de investimentos em infraestrutura da história do país, com forte participação do capital privado via concessões e PPPs. Defende reunificar o Ministério da Infraestrutura, modernizar a malha ferroviária com autorizações e concessões, expandir portos e aeroportos com mais participação privada e consolidar as hidrovias como corredor estratégico. Propõe também modernizar a gestão rodoviária com contratos de longo prazo e tecnologia de monitoramento, além de instituir uma política nacional de mobilidade urbana para expandir metrôs, trens e VLTs nas grandes regiões metropolitanas. Busca ainda simplificar o licenciamento ambiental e criar um regime especial para acelerar obras estratégicas de interesse nacional.</t>
         </is>
       </c>
       <c r="F90" s="4" t="inlineStr">
@@ -3243,7 +3339,7 @@
       </c>
       <c r="E91" s="4" t="inlineStr">
         <is>
-          <t>O plano defende um licenciamento ambiental com critérios técnicos e previsibilidade, sem travar o desenvolvimento econômico, além de combater com rigor a grilagem e o desmatamento ilegal com monitoramento por satélite. Propõe avançar no Novo Marco do Saneamento e melhorar a gestão de resíduos para universalizar água e esgoto. Defende transformar o potencial ambiental em riqueza, com bioeconomia, turismo sustentável e um ambiente seguro para comercializar créditos de carbono no mercado internacional. Por fim, propõe ampliar investimentos em prevenção a desastres climáticos e planejamento urbano para reduzir riscos de enchentes.</t>
+          <t>O plano defende um licenciamento ambiental com critérios técnicos e previsibilidade, sem travar o desenvolvimento econômico, além de combater com rigor a grilagem e o desmatamento ilegal com monitoramento por satélite. Propõe avançar na modernização do marco regulatório do saneamento e melhorar a gestão de resíduos para universalizar água e esgoto. Defende transformar o potencial ambiental em riqueza, com bioeconomia, turismo sustentável e um ambiente seguro para comercializar créditos de carbono no mercado internacional. Por fim, propõe ampliar investimentos em prevenção a desastres climáticos e planejamento urbano para reduzir riscos de enchentes.</t>
         </is>
       </c>
       <c r="F91" s="4" t="inlineStr">
@@ -3252,7 +3348,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="120" customHeight="1">
+    <row r="92" ht="135" customHeight="1">
       <c r="A92" s="2" t="inlineStr">
         <is>
           <t>30</t>
@@ -3275,12 +3371,12 @@
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
-          <t>O plano cria o programa Casas da Cidadania para oferecer, a cada família vulnerável, um plano individualizado de capacitação, trabalho e acesso à moradia. Propõe condicionar a permanência no Bolsa Família à busca por emprego ou qualificação, com um prêmio de R$5 mil para quem sai do programa e conquista autonomia. Defende unificar programas de transferência de renda, combater fraudes no CadÚnico e reformular o Minha Casa, Minha Vida para priorizar áreas com infraestrutura. Para a população em situação de rua, propõe proibir barracas em espaços públicos, ampliar moradias de interesse social e permitir internação involuntária de dependentes químicos. Também amplia a proteção a idosos, crianças e vítimas de violência doméstica.</t>
+          <t>O plano cria um programa municipal para oferecer, a cada família vulnerável, um plano individualizado de capacitação, trabalho e acesso à moradia. Propõe condicionar a permanência no programa federal de transferência de renda à busca por emprego ou qualificação, com um prêmio de R$5 mil para quem sai do programa e conquista autonomia. Defende unificar programas de transferência de renda, combater fraudes no cadastro de beneficiários e reformular o principal programa habitacional federal para priorizar áreas com infraestrutura. Para a população em situação de rua, propõe proibir barracas em espaços públicos, ampliar moradias de interesse social e permitir internação involuntária de dependentes químicos. Também amplia a proteção a idosos, crianças e vítimas de violência doméstica.</t>
         </is>
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>Casas da Cidadania para tirar famílias da pobreza pelo trabalho, Bolsa Família condicionado e prêmio para quem sai do programa.</t>
+          <t>Programa municipal tira famílias da pobreza pelo trabalho, transferência de renda condicionada e prêmio para quem sai do programa.</t>
         </is>
       </c>
     </row>
@@ -3467,12 +3563,12 @@
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
-          <t>O plano foca no que compete à União: financiar, avaliar, induzir e formar, já que não administra escolas de ensino fundamental. Propõe continuidade e fortalecimento da política de alfabetização na idade certa, com condicionalidade a resultados de avaliação externa e transparência dos dados por escola. Defende ampliação da rede federal de educação profissional integrada ao ensino médio e a programas de qualificação. A proposta central e mais inovadora é a PEC da Pesquisa, que transformaria pesquisadores de bolsistas em servidores públicos com carreira, salário e vínculo previdenciário, combatendo a fuga de cérebros formados com dinheiro público. Também prevê educação física de verdade nas escolas, com professor formado, carga horária mínima e avaliação de aptidão física dos estudantes.</t>
+          <t>O plano foca no que compete à União: financiar, avaliar, induzir e formar, já que não administra escolas de ensino fundamental. Propõe continuidade e fortalecimento da política de alfabetização na idade certa, com condicionalidade a resultados de avaliação externa e transparência dos dados por escola. Defende ampliação da rede federal de educação profissional integrada ao ensino médio e a programas de qualificação. A proposta central e mais inovadora é uma emenda constitucional para transformar pesquisadores hoje sustentados por bolsas em servidores públicos com carreira, salário e vínculo previdenciário, combatendo a fuga de cérebros formados com dinheiro público. Também prevê educação física de verdade nas escolas, com professor formado, carga horária mínima e avaliação de aptidão física dos estudantes.</t>
         </is>
       </c>
       <c r="F98" s="4" t="inlineStr">
         <is>
-          <t>Alfabetização com condicionalidade, PEC da Pesquisa para efetivar pesquisadores e educação física de verdade nas escolas.</t>
+          <t>Alfabetização com condicionalidade, emenda para efetivar pesquisadores como servidores e educação física de verdade nas escolas.</t>
         </is>
       </c>
     </row>
@@ -3499,12 +3595,12 @@
       </c>
       <c r="E99" s="4" t="inlineStr">
         <is>
-          <t>A proposta central é o Imposto Único Federal, um tributo sobre movimentação financeira (2% no débito e 2% no crédito) que substituiria nove tributos federais que incidem sobre folha, faturamento e produção, como a contribuição patronal, Cofins, CSLL, IPI e IOF. O limite de isenção do Imposto de Renda subiria para cinco salários mínimos (R$ 8.105 em 2026), isentando cerca de 85% da população, com tabela progressiva mantida acima do limite. A reforma prevê salvaguardas como devolução do tributo na exportação, blindagem da desoneração da folha, cláusula de revisão automática e restrições à circulação de dinheiro em espécie. A transição ocorreria em três etapas — convivência, repactuação federativa e desligamento dos tributos antigos — via Proposta de Emenda à Constituição. O plano detalha estudo de impacto com números de fontes oficiais, incluindo custo da isenção (R$ 266 bi/ano) e meta de arrecadação (R$ 1.828 bi/ano).</t>
+          <t>A proposta central é um tributo único federal sobre movimentação financeira (2% no débito e 2% no crédito) que substituiria nove tributos federais que incidem sobre folha, faturamento e produção, como a contribuição patronal, Cofins, CSLL, IPI e IOF. O limite de isenção do Imposto de Renda subiria para cinco salários mínimos (R$ 8.105 em 2026), isentando cerca de 85% da população, com tabela progressiva mantida acima do limite. A reforma prevê salvaguardas como devolução do tributo na exportação, blindagem da desoneração da folha, cláusula de revisão automática e restrições à circulação de dinheiro em espécie. A transição ocorreria em três etapas — convivência, repactuação federativa e desligamento dos tributos antigos — via Proposta de Emenda à Constituição. O plano detalha estudo de impacto com números de fontes oficiais, incluindo custo da isenção (R$ 266 bi/ano) e meta de arrecadação (R$ 1.828 bi/ano).</t>
         </is>
       </c>
       <c r="F99" s="4" t="inlineStr">
         <is>
-          <t>IUF substitui 9 tributos federais por tributo único sobre movimentação financeira; isenção do IR sobe a 5 salários mínimos.</t>
+          <t>Um tributo único substitui 9 tributos federais sobre movimentação financeira; isenção do IR sobe a 5 salários mínimos.</t>
         </is>
       </c>
     </row>
@@ -3531,12 +3627,12 @@
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
-          <t>O plano cria o conceito de "Saúde Única", integrando saúde humana, animal e ambiental, com veterinários nas equipes de vigilância municipal e programa nacional de vigilância de zoonoses (raiva, leishmaniose, leptospirose). Propõe atendimento veterinário público para famílias de baixa renda e integração de dados sanitários humanos e animais para detectar surtos cedo. Na atenção primária, defende expansão das equipes de saúde da família com financiamento estável e carreira para profissionais em regiões de difícil fixação. Cria fila nacional única e pública por procedimento cirúrgico e diagnóstico, com posição consultável pelo próprio paciente e mutirões contratualizados por resultado. Também prevê fortalecimento da produção nacional de medicamentos e imunizantes, inclusive veterinários, e plano de contingência para emergências sanitárias.</t>
+          <t>O plano integra saúde humana, animal e ambiental em uma só política, com veterinários nas equipes de vigilância municipal e programa nacional de vigilância de zoonoses (raiva, leishmaniose, leptospirose). Propõe atendimento veterinário público para famílias de baixa renda e integração de dados sanitários humanos e animais para detectar surtos cedo. Na atenção primária, defende expansão das equipes de saúde da família com financiamento estável e carreira para profissionais em regiões de difícil fixação. Cria fila nacional única e pública por procedimento cirúrgico e diagnóstico, com posição consultável pelo próprio paciente e mutirões contratualizados por resultado. Também prevê fortalecimento da produção nacional de medicamentos e imunizantes, inclusive veterinários, e plano de contingência para emergências sanitárias.</t>
         </is>
       </c>
       <c r="F100" s="4" t="inlineStr">
         <is>
-          <t>Saúde Única integra vigilância humana e animal; fila nacional pública de cirurgias; mais equipes de saúde da família com carreira estável.</t>
+          <t>Integração da vigilância humana e animal; fila nacional pública de cirurgias; mais equipes de saúde da família com carreira estável.</t>
         </is>
       </c>
     </row>
@@ -3563,16 +3659,16 @@
       </c>
       <c r="E101" s="4" t="inlineStr">
         <is>
-          <t>A política de segurança pública se organiza em cinco pilares sequenciais: isolar o comando das facções em presídios federais de segurança máxima, asfixiar o dinheiro do crime organizado via inteligência financeira, fechar fronteiras e portos, integrar as bases de dados de segurança (aplicando lei já existente) e prevenir com cadastro de infratores por maus-tratos a animais como alerta de violência doméstica. Propõe plebiscito para decidir se o Brasil adota modelo penitenciário de segurança máxima inspirado em El Salvador, mas ressalva que garantias individuais e devido processo são cláusulas pétreas e não podem ser suprimidas. Na defesa nacional, defende elevar o orçamento militar a 2% do PIB (PEC 55/2023), com 35% vinculado à modernização, recompor o soldo dos praças (hoje abaixo do salário mínimo) e emprego permanente das Forças Armadas na fronteira contra tráfico de armas e drogas, com regras de engajamento e prazos definidos.</t>
+          <t>A política de segurança pública se organiza em cinco pilares sequenciais: isolar o comando das facções em presídios federais de segurança máxima, asfixiar o dinheiro do crime organizado via inteligência financeira, fechar fronteiras e portos, integrar as bases de dados de segurança (aplicando lei já existente) e prevenir com cadastro de infratores por maus-tratos a animais como alerta de violência doméstica. Propõe plebiscito para decidir se o Brasil adota modelo penitenciário de segurança máxima inspirado em outros países, mas ressalva que garantias individuais e devido processo são cláusulas pétreas e não podem ser suprimidas. Na defesa nacional, defende elevar o orçamento militar a 2% do PIB, com 35% vinculado à modernização, recompor o soldo dos praças (hoje abaixo do salário mínimo) e emprego permanente das Forças Armadas na fronteira contra tráfico de armas e drogas, com regras de engajamento e prazos definidos.</t>
         </is>
       </c>
       <c r="F101" s="4" t="inlineStr">
         <is>
-          <t>Cinco pilares contra o crime organizado, presídio federal para líderes de facção e plebiscito sobre modelo penitenciário tipo El Salvador.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="120" customHeight="1">
+          <t>Cinco pilares contra o crime organizado, presídio federal para líderes de facção e plebiscito sobre modelo penitenciário mais rígido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="105" customHeight="1">
       <c r="A102" s="2" t="inlineStr">
         <is>
           <t>35</t>
@@ -3595,12 +3691,12 @@
       </c>
       <c r="E102" s="4" t="inlineStr">
         <is>
-          <t>O programa "Brasil nos Trilhos" propõe retomar e concluir corredores ferroviários de carga prioritários, com cronograma físico publicado, para reduzir a dependência do transporte rodoviário em distâncias continentais. Defende uso pleno do regime de autorização ferroviária para que o setor privado construa e opere ferrovias, cabendo ao Estado licenciar rapidamente e garantir estabilidade regulatória. Propõe integração planejada entre ferrovia e porto, além de maior uso de hidrovias e cabotagem. Prioriza investimentos por critério de custo logístico por tonelada transportada, publicado por corredor, e fiscalização efetiva dos contratos de concessão, com penalidades aplicadas.</t>
+          <t>O plano propõe retomar e concluir corredores ferroviários de carga prioritários, com cronograma físico publicado, para reduzir a dependência do transporte rodoviário em distâncias continentais. Defende uso pleno do regime de autorização ferroviária para que o setor privado construa e opere ferrovias, cabendo ao Estado licenciar rapidamente e garantir estabilidade regulatória. Propõe integração planejada entre ferrovia e porto, além de maior uso de hidrovias e cabotagem. Prioriza investimentos por critério de custo logístico por tonelada transportada, publicado por corredor, e fiscalização efetiva dos contratos de concessão, com penalidades aplicadas.</t>
         </is>
       </c>
       <c r="F102" s="4" t="inlineStr">
         <is>
-          <t>Programa Brasil nos Trilhos amplia ferrovias de carga, hidrovias e cabotagem, com fiscalização real das concessões, para baratear o frete.</t>
+          <t>Retomada de ferrovias de carga, mais hidrovias e cabotagem, com fiscalização real das concessões, para baratear o frete.</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3755,7 @@
       </c>
       <c r="E104" s="4" t="inlineStr">
         <is>
-          <t>O eixo de habitação propõe inverter a lógica da política atual: em vez do Estado escolher onde a pessoa mora, quem paga aluguel e comprova capacidade de pagamento por esse histórico teria acesso automático a financiamento habitacional com parcela equivalente ao aluguel, podendo escolher livremente o imóvel, novo ou usado, em qualquer cidade. Os juros viriam do direcionamento do FGTS e da poupança, redução do custo de originação e garantia pública parcial para quem não tem entrada. Prevê também titulação em massa em áreas urbanas consolidadas e assistência técnica gratuita para reforma. A meta declarada é reduzir o déficit habitacional medido pela Fundação João Pinheiro, com metas de cobertura ao longo do mandato.</t>
+          <t>O eixo de habitação propõe inverter a lógica da política atual: em vez do Estado escolher onde a pessoa mora, quem paga aluguel e comprova capacidade de pagamento por esse histórico teria acesso automático a financiamento habitacional com parcela equivalente ao aluguel, podendo escolher livremente o imóvel, novo ou usado, em qualquer cidade. Os juros viriam do direcionamento do FGTS e da poupança, redução do custo de originação e garantia pública parcial para quem não tem entrada. Prevê também titulação em massa em áreas urbanas consolidadas e assistência técnica gratuita para reforma. A meta declarada é reduzir o déficit habitacional medido por instituto oficial de pesquisa, com metas de cobertura ao longo do mandato.</t>
         </is>
       </c>
       <c r="F104" s="4" t="inlineStr">
@@ -3723,12 +3819,12 @@
       </c>
       <c r="E106" s="4" t="inlineStr">
         <is>
-          <t>A proposta central é a PEC da Pesquisa, que transformaria pesquisadores que hoje vivem de bolsa em servidores públicos com carreira, vínculo, previdência e salário compatível com sua qualificação, para reter no país profissionais formados com dinheiro público. A carreira teria ingresso por processo seletivo baseado em produção científica, fomento em todas as áreas sem lista de temas privilegiados, e cláusula de contrapartida com compromisso de permanência. Defende também financiamento estável e plurianual à pesquisa, para que não fique sujeito a contingenciamento, com fomento dirigido a sanidade animal, zoonoses e imunizantes veterinários, área em que o Brasil tem base instalada e subaproveitada.</t>
+          <t>A proposta central é uma emenda constitucional para transformar pesquisadores que hoje vivem de bolsa em servidores públicos com carreira, vínculo, previdência e salário compatível com sua qualificação, para reter no país profissionais formados com dinheiro público. A carreira teria ingresso por processo seletivo baseado em produção científica, fomento em todas as áreas sem lista de temas privilegiados, e cláusula de contrapartida com compromisso de permanência. Defende também financiamento estável e plurianual à pesquisa, para que não fique sujeito a contingenciamento, com fomento dirigido a sanidade animal, zoonoses e imunizantes veterinários, área em que o Brasil tem base instalada e subaproveitada.</t>
         </is>
       </c>
       <c r="F106" s="4" t="inlineStr">
         <is>
-          <t>PEC da Pesquisa transforma bolsistas em servidores com carreira e salário, para reter cientistas formados com dinheiro público no Brasil.</t>
+          <t>Emenda constitucional transforma bolsistas em servidores com carreira e salário, para reter cientistas formados com dinheiro público.</t>
         </is>
       </c>
     </row>
@@ -3755,7 +3851,7 @@
       </c>
       <c r="E107" s="4" t="inlineStr">
         <is>
-          <t>O plano defende zerar o custo tributário de contratar, com a extinção da contribuição patronal sobre a folha de pagamento pelo Imposto Único Federal, apostando que a informalidade migrará para o trabalho formal à medida que o vínculo ficar mais barato. Propõe simplificar obrigações acessórias trabalhistas e previdenciárias em envio único, com prazos legais de resposta da administração e responsabilização de servidores e dirigentes por atrasos injustificados. Para pequenos negócios, defende revisão do enquadramento do MEI, abertura e baixa de empresa em ambiente único digital, e tratamento favorecido efetivo nas compras públicas. Prevê ainda programa de qualificação profissional vinculado à demanda real de contratação na região, e não ao catálogo pronto das instituições de ensino.</t>
+          <t>O plano defende zerar o custo tributário de contratar, com a extinção da contribuição patronal sobre a folha de pagamento por meio da reforma tributária proposta, apostando que a informalidade migrará para o trabalho formal à medida que o vínculo ficar mais barato. Propõe simplificar obrigações acessórias trabalhistas e previdenciárias em envio único, com prazos legais de resposta da administração e responsabilização de servidores e dirigentes por atrasos injustificados. Para pequenos negócios, defende revisão do enquadramento do MEI, abertura e baixa de empresa em ambiente único digital, e tratamento favorecido efetivo nas compras públicas. Prevê ainda programa de qualificação profissional vinculado à demanda real de contratação na região, e não ao catálogo pronto das instituições de ensino.</t>
         </is>
       </c>
       <c r="F107" s="4" t="inlineStr">
@@ -3819,7 +3915,7 @@
       </c>
       <c r="E109" s="4" t="inlineStr">
         <is>
-          <t>O plano trata bem-estar animal e agronegócio como agenda complementar, defendendo que padrão sanitário, rastreabilidade e bem-estar animal são vantagem competitiva na exportação. Propõe recompor o serviço veterinário oficial com concurso e carreira, manter e ampliar status sanitários internacionais e responder rapidamente a focos sanitários com protocolo pré-acordado. Critica o cronograma do Plano Nacional de Identificação de Bovinos e Búfalos (concluído só em 2032) por ficar seis anos atrás da exigência europeia de rastreabilidade (2026), propondo antecipação voluntária apoiada pela União, especialmente para pequenos produtores. Defende também crédito simplificado e assistência técnica para agricultura familiar, além de compras públicas de alimentação escolar priorizando produção local.</t>
+          <t>O plano trata bem-estar animal e agronegócio como agenda complementar, defendendo que padrão sanitário, rastreabilidade e bem-estar animal são vantagem competitiva na exportação. Propõe recompor o serviço veterinário oficial com concurso e carreira, manter e ampliar status sanitários internacionais e responder rapidamente a focos sanitários com protocolo pré-acordado. Critica o cronograma federal de identificação de bovinos e búfalos (concluído só em 2032) por ficar seis anos atrás da exigência europeia de rastreabilidade (2026), propondo antecipação voluntária apoiada pela União, especialmente para pequenos produtores. Defende também crédito simplificado e assistência técnica para agricultura familiar, além de compras públicas de alimentação escolar priorizando produção local.</t>
         </is>
       </c>
       <c r="F109" s="4" t="inlineStr">
@@ -3915,7 +4011,7 @@
       </c>
       <c r="E112" s="4" t="inlineStr">
         <is>
-          <t>O plano prevê a modernização do SUS, mantendo-o universal, mas tornando-o mais preventivo, digital e organizado por prioridade clínica em vez de fila cronológica. Propõe um Sistema Nacional de Acesso e Regulação Inteligente para reduzir filas, fortalecimento da Atenção Primária, redes nacionais para infarto, AVC e câncer, e programas específicos para saúde da mulher, infância, saúde mental e longevidade. Também busca soberania sanitária, com produção nacional de medicamentos, vacinas e terapias avançadas, e maior uso de dados e inteligência artificial na gestão hospitalar. Estabelece metas nacionais para 2030 em diversas áreas, como redução de mortalidade materna e cardiovascular e ampliação da cobertura vacinal.</t>
+          <t>O plano prevê a modernização do SUS, mantendo-o universal, mas tornando-o mais preventivo, digital e organizado por prioridade clínica em vez de fila cronológica. Propõe um sistema nacional de regulação de acesso baseado em inteligência artificial para reduzir filas, fortalecimento da Atenção Primária, redes nacionais para infarto, AVC e câncer, e programas específicos para saúde da mulher, infância, saúde mental e longevidade. Também busca soberania sanitária, com produção nacional de medicamentos, vacinas e terapias avançadas, e maior uso de dados e inteligência artificial na gestão hospitalar. Estabelece metas nacionais para 2030 em diversas áreas, como redução de mortalidade materna e cardiovascular e ampliação da cobertura vacinal.</t>
         </is>
       </c>
       <c r="F112" s="4" t="inlineStr">
@@ -3947,7 +4043,7 @@
       </c>
       <c r="E113" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe a criação do Ministério da Segurança Pública e de um Sistema Integrado de Proteção à Soberania Nacional, com nova legislação que classifica facções e milícias como organizações terroristas domésticas, prevendo penas mínimas elevadas e regime prisional mais rígido para lideranças criminosas. Prevê a asfixia financeira do crime organizado, com inversão do ônus da prova patrimonial e perdimento acelerado de bens, além de reforço no controle de fronteiras, portos e da Amazônia. Propõe redução da maioridade penal para 16 anos em crimes graves, criação de secretaria nacional de segurança da mulher e da criança, e combate à corrupção com um sistema nacional anticorrupção. A experiência de segurança pública do governo de Goiás é citada como modelo a ser replicado nacionalmente.</t>
+          <t>O plano propõe a criação do Ministério da Segurança Pública e de um sistema integrado de proteção à soberania nacional, com nova legislação que classifica facções e milícias como organizações terroristas domésticas, prevendo penas mínimas elevadas e regime prisional mais rígido para lideranças criminosas. Prevê a asfixia financeira do crime organizado, com inversão do ônus da prova patrimonial e perdimento acelerado de bens, além de reforço no controle de fronteiras, portos e da Amazônia. Propõe redução da maioridade penal para 16 anos em crimes graves, criação de secretaria nacional de segurança da mulher e da criança, e combate à corrupção com um sistema nacional anticorrupção. A experiência bem-sucedida de um governo estadual em segurança pública é citada como modelo a ser replicado nacionalmente.</t>
         </is>
       </c>
       <c r="F113" s="4" t="inlineStr">
@@ -4043,7 +4139,7 @@
       </c>
       <c r="E116" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe um Sistema Nacional de Gestão Social Integrada, unificando Cadastro Único, SUAS, saúde, educação e trabalho para acompanhar famílias vulneráveis de forma coordenada. Mantém programas de transferência de renda, mas cria regras de transição para quem ingressa no mercado de trabalho, além de um Plano Nacional de Emancipação Social com qualificação, crédito e intermediação de emprego. Estabelece prioridade absoluta para crianças e adolescentes, com ações voltadas à primeira infância, combate à fome, proteção contra violências e ao sistema socioeducativo. Também prevê políticas para pessoas idosas, pessoas com deficiência e população em situação de rua.</t>
+          <t>O plano propõe um sistema nacional de gestão social integrada, unificando Cadastro Único, SUAS, saúde, educação e trabalho para acompanhar famílias vulneráveis de forma coordenada. Mantém programas de transferência de renda, mas cria regras de transição para quem ingressa no mercado de trabalho, além de um plano nacional de emancipação social com qualificação, crédito e intermediação de emprego. Estabelece prioridade absoluta para crianças e adolescentes, com ações voltadas à primeira infância, combate à fome, proteção contra violências e ao sistema socioeducativo. Também prevê políticas para pessoas idosas, pessoas com deficiência e população em situação de rua.</t>
         </is>
       </c>
       <c r="F116" s="4" t="inlineStr">
@@ -4171,7 +4267,7 @@
       </c>
       <c r="E120" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe um "Governo Transformador" baseado em método: priorização nacional por missões, escolha de dirigentes por competência e integridade, e um Centro de Governo para coordenar ministérios e monitorar resultados. Defende reformas do sistema político, incluindo o fim da reeleição no Executivo e adoção de sistema distrital misto, além de maior transparência nas emendas parlamentares e no orçamento. Propõe digitalização do Estado, com identidade digital única para o cidadão, avaliação periódica de políticas públicas e um Sistema Nacional Anticorrupção. A execução será monitorada por um Plano Plurianual orientado a missões e por um painel público de indicadores, o "Painel Brasil 2030".</t>
+          <t>O plano propõe um modelo de governo baseado em método: priorização nacional por missões, escolha de dirigentes por competência e integridade, e um centro de governo para coordenar ministérios e monitorar resultados. Defende reformas do sistema político, incluindo o fim da reeleição no Executivo e adoção de sistema distrital misto, além de maior transparência nas emendas parlamentares e no orçamento. Propõe digitalização do Estado, com identidade digital única para o cidadão, avaliação periódica de políticas públicas e um sistema nacional anticorrupção. A execução será monitorada por um Plano Plurianual orientado a missões e por um painel público de indicadores de resultados.</t>
         </is>
       </c>
       <c r="F120" s="4" t="inlineStr">
@@ -4203,7 +4299,7 @@
       </c>
       <c r="E121" s="4" t="inlineStr">
         <is>
-          <t>O plano trata o agronegócio como plataforma de liderança global do Brasil em alimentos, bioenergia e biotecnologia, priorizando ganhos de produtividade nas áreas já abertas em vez de expansão da fronteira agrícola. Propõe uma nova arquitetura de financiamento com foco em seguro rural, garantias e um Plano Safra plurianual, além de fortalecer a Embrapa e reduzir a dependência externa de fertilizantes. Defende investimentos em logística (ferrovias, hidrovias e armazenagem), regularização fundiária e ambiental, e abertura de novos mercados internacionais para os produtos brasileiros. Também propõe transformar a sustentabilidade em vantagem comercial, com rastreabilidade e um selo de sustentabilidade brasileiro.</t>
+          <t>O plano trata o agronegócio como plataforma de liderança global do Brasil em alimentos, bioenergia e biotecnologia, priorizando ganhos de produtividade nas áreas já abertas em vez de expansão da fronteira agrícola. Propõe uma nova arquitetura de financiamento com foco em seguro rural, garantias e um plano de crédito agrícola plurianual, além de fortalecer a Embrapa e reduzir a dependência externa de fertilizantes. Defende investimentos em logística (ferrovias, hidrovias e armazenagem), regularização fundiária e ambiental, e abertura de novos mercados internacionais para os produtos brasileiros. Também propõe transformar a sustentabilidade em vantagem comercial, com rastreabilidade e um selo de sustentabilidade brasileiro.</t>
         </is>
       </c>
       <c r="F121" s="4" t="inlineStr">
@@ -4235,7 +4331,7 @@
       </c>
       <c r="E122" s="4" t="inlineStr">
         <is>
-          <t>O plano defende a educação como prioridade absoluta do Estado, com foco na alfabetização na idade certa, valorização e formação contínua dos professores e redução das desigualdades educacionais. Propõe um Novo Ensino Médio integrado a empreendedorismo, educação financeira, gestão da emoção e tecnologia, além de universidades voltadas à pesquisa aplicada, inovação e geração de patentes. Cria o programa Brasil Neuroinclusivo para acolher estudantes com autismo, TDAH e dislexia, com metodologia pedagógica baseada em provocar perguntas, desafiar o pensamento e elogiar a participação. Prevê também escolas de tempo integral transformadas em 'clubes de desenvolvimento humano', com esportes, arte e debate.</t>
+          <t>O plano defende a educação como prioridade absoluta do Estado, com foco na alfabetização na idade certa, valorização e formação contínua dos professores e redução das desigualdades educacionais. Propõe um Novo Ensino Médio integrado a empreendedorismo, educação financeira, gestão da emoção e tecnologia, além de universidades voltadas à pesquisa aplicada, inovação e geração de patentes. Cria um programa nacional de acolhimento neuroinclusivo para estudantes com autismo, TDAH e dislexia, com metodologia pedagógica baseada em provocar perguntas, desafiar o pensamento e elogiar a participação. Prevê também escolas de tempo integral transformadas em 'clubes de desenvolvimento humano', com esportes, arte e debate.</t>
         </is>
       </c>
       <c r="F122" s="4" t="inlineStr">
@@ -4267,12 +4363,12 @@
       </c>
       <c r="E123" s="4" t="inlineStr">
         <is>
-          <t>O programa econômico combina responsabilidade fiscal (déficit próximo de zero, controle de gastos, redução gradual da dívida) com simplificação tributária e reforma administrativa do Estado. Defende forte estímulo ao empreendedorismo, com 10 mil escolas de empreendedorismo, Banco do Empreendedor, meta de 10 milhões de novos empreendedores e um programa de 10 mil novas indústrias, incluindo semicondutores, farmacêutica e terras raras. Propõe também cinco Corredores Estratégicos de Exportação e Zonas de Processamento de Exportação para ampliar o comércio exterior brasileiro.</t>
+          <t>O programa econômico combina responsabilidade fiscal (déficit próximo de zero, controle de gastos, redução gradual da dívida) com simplificação tributária e reforma administrativa do Estado. Defende forte estímulo ao empreendedorismo, com 10 mil escolas de empreendedorismo, um banco público de apoio ao empreendedor, meta de 10 milhões de novos empreendedores e um programa de 10 mil novas indústrias, incluindo semicondutores, farmacêutica e terras raras. Propõe também cinco corredores estratégicos de exportação e zonas de processamento de exportação para ampliar o comércio exterior brasileiro.</t>
         </is>
       </c>
       <c r="F123" s="4" t="inlineStr">
         <is>
-          <t>Economia: responsabilidade fiscal, simplificação tributária, Banco do Empreendedor e meta de 10 milhões de novos empreendedores no Brasil.</t>
+          <t>Economia: responsabilidade fiscal, simplificação tributária, banco de apoio ao empreendedor e meta de 10 milhões de novos empreendedores.</t>
         </is>
       </c>
     </row>
@@ -4299,16 +4395,16 @@
       </c>
       <c r="E124" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe transformar o Brasil na maior plataforma pública de telemedicina do mundo (Tele Saúde Brasil), usando inteligência artificial para triagem e metas de atendimento digital em até 30 minutos, desafogando o SUS. Fortalece a atenção primária, a modernização do SUS e cria um Programa Nacional de Saúde Mental com foco na prevenção da ansiedade, automutilação e suicídio. Institui também o projeto Sociedade Está Abraçando (SEA), de prevenção e detecção precoce do câncer, inspirado no modelo do Hospital de Amor de Barretos.</t>
+          <t>O plano propõe transformar o Brasil na maior plataforma pública de telemedicina do mundo, usando inteligência artificial para triagem e metas de atendimento digital em até 30 minutos, desafogando o SUS. Fortalece a atenção primária, a modernização do SUS e cria um Programa Nacional de Saúde Mental com foco na prevenção da ansiedade, automutilação e suicídio. Institui também um projeto de prevenção e detecção precoce do câncer, inspirado em centros de referência no tratamento oncológico.</t>
         </is>
       </c>
       <c r="F124" s="4" t="inlineStr">
         <is>
-          <t>Saúde: telemedicina para desafogar o SUS, Programa de Saúde Mental e projeto SEA de prevenção e detecção precoce do câncer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="90" customHeight="1">
+          <t>Saúde: telemedicina para desafogar o SUS, Programa de Saúde Mental e projeto de prevenção e detecção precoce do câncer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="75" customHeight="1">
       <c r="A125" s="2" t="inlineStr">
         <is>
           <t>70</t>
@@ -4331,12 +4427,12 @@
       </c>
       <c r="E125" s="4" t="inlineStr">
         <is>
-          <t>O plano cria o Programa FATO (Força de Alerta Total), que integra Polícia Federal, Militar, Civil e uma nova força municipal (FOCO) em um centro nacional de inteligência com IA, drones e câmeras inteligentes. Propõe recriação do Ministério da Segurança Pública, combate estruturado ao crime organizado com foco nas finanças das facções, e reforço das fronteiras com Forças Armadas. Inclui também o Programa Mulheres Vivas, de prevenção ao feminicídio, e reforma do sistema penitenciário com foco em ressocialização.</t>
+          <t>O plano cria um programa que integra Polícia Federal, Militar, Civil e uma nova força municipal em um centro nacional de inteligência com IA, drones e câmeras inteligentes. Propõe recriação do Ministério da Segurança Pública, combate estruturado ao crime organizado com foco nas finanças das facções, e reforço das fronteiras com Forças Armadas. Inclui também um programa de prevenção ao feminicídio, e reforma do sistema penitenciário com foco em ressocialização.</t>
         </is>
       </c>
       <c r="F125" s="4" t="inlineStr">
         <is>
-          <t>Segurança: Programa FATO integra polícias e a força municipal FOCO com IA e drones, e recria o Ministério da Segurança.</t>
+          <t>Segurança: programa integra polícias e uma nova força municipal com IA e drones, e recria o Ministério da Segurança Pública.</t>
         </is>
       </c>
     </row>
@@ -4363,12 +4459,12 @@
       </c>
       <c r="E126" s="4" t="inlineStr">
         <is>
-          <t>O programa propõe a duplicação das principais rodovias federais para reduzir acidentes e mortes no trânsito, além de um grande programa nacional de integração logística envolvendo rodovias, ferrovias, hidrovias, portos e aeroportos. Cria o projeto BEE (Brasil Empreendedor nas Estradas), que instala polos de comércio popular a cada 10-15 km ao longo das rodovias, com energia solar, áreas de descanso e apoio a pequenos produtores e agricultores familiares. Também prevê ampliação das concessões e parcerias público-privadas para acelerar obras de infraestrutura.</t>
+          <t>O programa propõe a duplicação das principais rodovias federais para reduzir acidentes e mortes no trânsito, além de um grande programa nacional de integração logística envolvendo rodovias, ferrovias, hidrovias, portos e aeroportos. Cria um projeto que instala polos de comércio popular a cada 10-15 km ao longo das rodovias, com energia solar, áreas de descanso e apoio a pequenos produtores e agricultores familiares. Também prevê ampliação das concessões e parcerias público-privadas para acelerar obras de infraestrutura.</t>
         </is>
       </c>
       <c r="F126" s="4" t="inlineStr">
         <is>
-          <t>Transporte: duplicação de rodovias, integração logística nacional e o projeto BEE, com polos de comércio a cada 10-15 km nas estradas.</t>
+          <t>Transporte: duplicação de rodovias, integração logística nacional e polos de comércio a cada 10-15 km ao longo das estradas.</t>
         </is>
       </c>
     </row>
@@ -4395,12 +4491,12 @@
       </c>
       <c r="E127" s="4" t="inlineStr">
         <is>
-          <t>O plano quer transformar o Brasil em potência mundial de energia limpa (PENER-BR), com hidrogênio verde, solar, eólica e energia oceânica, buscando 90% de matriz limpa até 2040. Cria o programa Floresta Viva-BR, com detecção de incêndios por satélites e IA, drones de combate ao fogo e o Programa Amazônia Viva, que busca gerar renda para ribeirinhos como forma de proteção ambiental. Propõe também mercado de carbono, pagamento por serviços ambientais aos produtores que preservam vegetação nativa, e industrialização responsável de terras raras (Petra-BR).</t>
+          <t>O plano quer transformar o Brasil em potência mundial de energia limpa, com hidrogênio verde, solar, eólica e energia oceânica, buscando 90% de matriz limpa até 2040. Cria um programa de detecção de incêndios por satélites e IA, com drones de combate ao fogo, além de uma iniciativa voltada a gerar renda para ribeirinhos como forma de proteção ambiental. Propõe também mercado de carbono, pagamento por serviços ambientais aos produtores que preservam vegetação nativa, e industrialização responsável de terras raras.</t>
         </is>
       </c>
       <c r="F127" s="4" t="inlineStr">
         <is>
-          <t>Meio Ambiente: energia limpa (PENER-BR), Floresta Viva-BR contra incêndios com IA e drones, e renda para ribeirinhos preservarem a Amazônia.</t>
+          <t>Meio Ambiente: energia limpa, combate a incêndios com IA e drones, e renda para ribeirinhos preservarem a Amazônia.</t>
         </is>
       </c>
     </row>
@@ -4427,12 +4523,12 @@
       </c>
       <c r="E128" s="4" t="inlineStr">
         <is>
-          <t>O plano cria o Projeto Mulheres Vivas, de proteção à vida e autonomia econômica das mulheres, com prevenção ao feminicídio, combate à desigualdade salarial e no crédito, e indicação de mulheres para o STF. Propõe desenvolvimento regional equilibrado, com Fundo Nacional de Desenvolvimento Regional, cinturões de proteína e cidades médias como polos de crescimento. Transforma o Bolsa Família em incentivo ao empreendedorismo e à formalização, e amplia programas de inclusão produtiva para famílias vulneráveis, unindo assistência com autonomia.</t>
+          <t>O plano cria um projeto de proteção à vida e autonomia econômica das mulheres, com prevenção ao feminicídio, combate à desigualdade salarial e no crédito, e indicação de mulheres para o STF. Propõe desenvolvimento regional equilibrado, com fundo nacional de desenvolvimento regional, cinturões de proteína e cidades médias como polos de crescimento. Transforma o principal programa de transferência de renda em incentivo ao empreendedorismo e à formalização, e amplia programas de inclusão produtiva para famílias vulneráveis, unindo assistência com autonomia.</t>
         </is>
       </c>
       <c r="F128" s="4" t="inlineStr">
         <is>
-          <t>Desenvolvimento Social: Programa Mulheres Vivas, combate à desigualdade salarial e o Bolsa Família como incentivo ao empreendedorismo.</t>
+          <t>Desenvolvimento Social: proteção às mulheres, combate à desigualdade salarial e renda como incentivo ao empreendedorismo e formalização.</t>
         </is>
       </c>
     </row>
@@ -4459,12 +4555,12 @@
       </c>
       <c r="E129" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe uma diplomacia econômica ativa, com o programa Embaixadas Empreendedoras (PEE), redistribuindo diplomatas para mercados emergentes como Índia e China, criando feiras internacionais do Brasil e uma rede de 'influenciadores embaixadores' e mulheres brasileiras no exterior para promover produtos nacionais. Eleva o Ministério das Relações Exteriores, propondo o título de Secretário de Estado. Defende ainda um Plano de Combate Mundial da Fome, com fundo internacional financiado por parte do comércio global e da indústria de armamentos.</t>
+          <t>O plano propõe uma diplomacia econômica ativa, redistribuindo diplomatas para mercados emergentes como Índia e China, criando feiras internacionais do Brasil e uma rede de 'influenciadores embaixadores' e mulheres brasileiras no exterior para promover produtos nacionais. Eleva o Ministério das Relações Exteriores, propondo o título de Secretário de Estado. Defende ainda um plano de combate mundial à fome, com fundo internacional financiado por parte do comércio global e da indústria de armamentos.</t>
         </is>
       </c>
       <c r="F129" s="4" t="inlineStr">
         <is>
-          <t>Relações Internacionais: diplomacia econômica ativa (PEE), embaixadas empreendedoras e fundo mundial de combate à fome.</t>
+          <t>Relações Internacionais: diplomacia econômica ativa, embaixadas empreendedoras e fundo mundial de combate à fome.</t>
         </is>
       </c>
     </row>
@@ -4491,12 +4587,12 @@
       </c>
       <c r="E130" s="4" t="inlineStr">
         <is>
-          <t>O plano trata a inteligência artificial como infraestrutura estratégica de Estado, com marco legal para IA, incentivo a startups universitárias e produção de patentes. Cria o programa Petra-BR para mapear e industrializar terras raras e minerais estratégicos, evitando a exportação apenas de matéria-prima. Propõe também polos industriais de semicondutores, biotecnologia e robótica, além de soberania digital e proteção de dados, buscando transformar universidades em centros de inovação conectados ao setor produtivo.</t>
+          <t>O plano trata a inteligência artificial como infraestrutura estratégica de Estado, com marco legal para IA, incentivo a startups universitárias e produção de patentes. Cria um programa para mapear e industrializar terras raras e minerais estratégicos, evitando a exportação apenas de matéria-prima. Propõe também polos industriais de semicondutores, biotecnologia e robótica, além de soberania digital e proteção de dados, buscando transformar universidades em centros de inovação conectados ao setor produtivo.</t>
         </is>
       </c>
       <c r="F130" s="4" t="inlineStr">
         <is>
-          <t>Ciência e Tecnologia: marco legal para IA, industrialização de terras raras (Petra-BR) e universidades como centros de inovação e patentes.</t>
+          <t>Ciência e Tecnologia: marco legal para IA, industrialização de terras raras e universidades como centros de inovação e patentes.</t>
         </is>
       </c>
     </row>
@@ -4523,12 +4619,12 @@
       </c>
       <c r="E131" s="4" t="inlineStr">
         <is>
-          <t>O plano cria a Secretaria/Ministério do Empreendedorismo e da Economia Distribuída, para preparar o país diante da automação e da inteligência artificial, com Escolas de Empreendedorismo, Banco do Empreendedor e crédito progressivo para pequenos negócios. Propõe programa de primeiro emprego para jovens, com incentivos fiscais para contratação, e amplia o cooperativismo (BCOO) para dobrar cooperados de 26 para 54 milhões. Não há um capítulo específico sobre reforma previdenciária no documento.</t>
+          <t>O plano cria a Secretaria/Ministério do Empreendedorismo e da Economia Distribuída, para preparar o país diante da automação e da inteligência artificial, com escolas de empreendedorismo, um banco público de apoio ao empreendedor e crédito progressivo para pequenos negócios. Propõe programa de primeiro emprego para jovens, com incentivos fiscais para contratação, e amplia o cooperativismo para dobrar cooperados de 26 para 54 milhões. Não há um capítulo específico sobre reforma previdenciária no documento.</t>
         </is>
       </c>
       <c r="F131" s="4" t="inlineStr">
         <is>
-          <t>Trabalho e Previdência: Ministério do Empreendedorismo, Banco do Empreendedor e programa de primeiro emprego para jovens brasileiros.</t>
+          <t>Trabalho e Previdência: Ministério do Empreendedorismo, banco de apoio ao empreendedor e programa de primeiro emprego para jovens.</t>
         </is>
       </c>
     </row>
@@ -4555,12 +4651,12 @@
       </c>
       <c r="E132" s="4" t="inlineStr">
         <is>
-          <t>O plano propõe mudar o regime de governo para semipresidencialismo, com Primeiro-Ministro escolhido pela maioria parlamentar, além de mandato de oito anos para ministros do STF. Defende um Estado digital, com metas para todos os ministérios, uso de inteligência artificial contra desperdícios e corrupção, e o programa Sociedade Está de Olho (SEO) de controle social dos gastos públicos. Propõe também reforma administrativa, simplificação tributária e reforma do sistema político para reduzir a fragmentação partidária.</t>
+          <t>O plano propõe mudar o regime de governo para semipresidencialismo, com Primeiro-Ministro escolhido pela maioria parlamentar, além de mandato de oito anos para ministros do STF. Defende um Estado digital, com metas para todos os ministérios, uso de inteligência artificial contra desperdícios e corrupção, e um programa de controle social dos gastos públicos. Propõe também reforma administrativa, simplificação tributária e reforma do sistema político para reduzir a fragmentação partidária.</t>
         </is>
       </c>
       <c r="F132" s="4" t="inlineStr">
         <is>
-          <t>Gestão Pública: semipresidencialismo, mandato de 8 anos no STF, governo digital e IA contra corrupção via o programa Sociedade Está de Olho.</t>
+          <t>Gestão Pública: semipresidencialismo, mandato de 8 anos no STF, governo digital e IA contra corrupção e controle social dos gastos.</t>
         </is>
       </c>
     </row>
@@ -4587,12 +4683,12 @@
       </c>
       <c r="E133" s="4" t="inlineStr">
         <is>
-          <t>O plano quer dobrar a produção agropecuária brasileira em 8 a 10 anos, com o programa Brasil Oásis para revolucionar o Semiárido por meio de irrigação inteligente, fruticultura e agroindústria. Propõe agricultura 4.0 com drones e IA, fortalecimento do pequeno produtor e do cooperativismo (meta de dobrar cooperados para 50 milhões), além do Agroindústria Brasil, com 10 mil novas agroindústrias e 100 usinas de etanol de milho. Amplia também o seguro rural e a abertura de mercados internacionais para o agronegócio.</t>
+          <t>O plano quer dobrar a produção agropecuária brasileira em 8 a 10 anos, com um programa para revolucionar o Semiárido por meio de irrigação inteligente, fruticultura e agroindústria. Propõe agricultura 4.0 com drones e IA, fortalecimento do pequeno produtor e do cooperativismo (meta de dobrar cooperados para 50 milhões), além de um programa de incentivo à agroindústria, com 10 mil novas agroindústrias e 100 usinas de etanol de milho. Amplia também o seguro rural e a abertura de mercados internacionais para o agronegócio.</t>
         </is>
       </c>
       <c r="F133" s="4" t="inlineStr">
         <is>
-          <t>Agricultura: dobrar a produção em 10 anos, revolução no Semiárido (Brasil Oásis), 10 mil agroindústrias e mais cooperativismo no campo.</t>
+          <t>Agricultura: dobrar a produção em 10 anos, revolução no Semiárido, 10 mil agroindústrias e mais cooperativismo no campo.</t>
         </is>
       </c>
     </row>
@@ -4619,12 +4715,12 @@
       </c>
       <c r="E134" s="4" t="inlineStr">
         <is>
-          <t>O programa defende educação pública, gratuita e laica em todos os níveis, com fim do lucro na educação e da privatização do ensino, incluindo estatização progressiva de conglomerados educacionais e anistia das dívidas do Fies. Propõe fim do vestibular e de qualquer processo seletivo, garantindo livre acesso à universidade e a cursos técnicos. Defende a revogação do Novo Ensino Médio, a destinação de pelo menos 10% do PIB à educação pública e um programa de erradicação do analfabetismo. Também prevê recomposição orçamentária das universidades e institutos federais, com bolsas, moradia estudantil e restaurante universitário, além de valorização salarial dos profissionais da educação e fim da terceirização.</t>
+          <t>O programa defende educação pública, gratuita e laica em todos os níveis, com fim do lucro na educação e da privatização do ensino, incluindo estatização progressiva de conglomerados educacionais e anistia das dívidas de financiamento estudantil. Propõe fim do vestibular e de qualquer processo seletivo, garantindo livre acesso à universidade e a cursos técnicos. Defende a revogação da atual reforma do ensino médio, a destinação de pelo menos 10% do PIB à educação pública e um programa de erradicação do analfabetismo. Também prevê recomposição orçamentária das universidades e institutos federais, com bolsas, moradia estudantil e restaurante universitário, além de valorização salarial dos profissionais da educação e fim da terceirização.</t>
         </is>
       </c>
       <c r="F134" s="4" t="inlineStr">
         <is>
-          <t>Educação 100% pública e gratuita em todos os níveis, sem vestibular, com 10% do PIB para o ensino e fim das dívidas do Fies.</t>
+          <t>Educação 100% pública e gratuita em todos os níveis, sem vestibular, com 10% do PIB para o ensino e fim das dívidas estudantis.</t>
         </is>
       </c>
     </row>
@@ -4651,7 +4747,7 @@
       </c>
       <c r="E135" s="4" t="inlineStr">
         <is>
-          <t>O programa propõe elevar em 100% o salário mínimo e reduzir a jornada de trabalho para 30 horas semanais sem redução salarial, encerrando a escala 6x1. Defende a suspensão do pagamento de juros da dívida pública, seguida de auditoria cidadã, e a nacionalização do sistema bancário sob controle dos trabalhadores. Propõe uma reforma tributária progressiva, com isenção de imposto de renda para trabalhadores e taxação de grandes fortunas, além do fim do Arcabouço Fiscal. A economia seria planificada de forma democrática, com controle público dos setores estratégicos e forte intervenção estatal para reduzir a desigualdade.</t>
+          <t>O programa propõe elevar em 100% o salário mínimo e reduzir a jornada de trabalho para 30 horas semanais sem redução salarial, encerrando a escala 6x1. Defende a suspensão do pagamento de juros da dívida pública, seguida de auditoria cidadã, e a nacionalização do sistema bancário sob controle dos trabalhadores. Propõe uma reforma tributária progressiva, com isenção de imposto de renda para trabalhadores e taxação de grandes fortunas, além do fim das atuais regras fiscais de controle de gastos públicos. A economia seria planificada de forma democrática, com controle público dos setores estratégicos e forte intervenção estatal para reduzir a desigualdade.</t>
         </is>
       </c>
       <c r="F135" s="4" t="inlineStr">
@@ -4747,7 +4843,7 @@
       </c>
       <c r="E138" s="4" t="inlineStr">
         <is>
-          <t>O programa defende a estatização das empresas de transporte coletivo, com fim das concessões e cartéis privados de ônibus, substituídos por empresas públicas municipais e estaduais. Propõe a transição progressiva para a tarifa zero no transporte urbano e intermunicipal, tratando o transporte como direito e não como negócio. Defende também a reestatização integral da CBTU e um Plano Nacional de Malha Ferroviária e Metroviária, com investimento prioritário em trens, metrôs e VLTs elétricos.</t>
+          <t>O programa defende a estatização das empresas de transporte coletivo, com fim das concessões e cartéis privados de ônibus, substituídos por empresas públicas municipais e estaduais. Propõe a transição progressiva para a tarifa zero no transporte urbano e intermunicipal, tratando o transporte como direito e não como negócio. Defende também a reestatização integral da CBTU e um amplo programa de expansão da malha ferroviária e metroviária, com investimento prioritário em trens, metrôs e VLTs elétricos.</t>
         </is>
       </c>
       <c r="F138" s="4" t="inlineStr">
@@ -4907,7 +5003,7 @@
       </c>
       <c r="E143" s="4" t="inlineStr">
         <is>
-          <t>O programa propõe o fim imediato da escala 6x1 e a redução da jornada de trabalho para 30 horas semanais sem redução salarial, além de aumento de 100% do salário mínimo. Defende a revogação das reformas trabalhista e previdenciária e o fim da terceirização irrestrita, com regulamentação rigorosa do trabalho por aplicativos, garantindo remuneração mínima e proteção previdenciária. Propõe a criação de Frentes Emergenciais de Trabalho, com empregos públicos diretos em obras de infraestrutura, moradia e saneamento, além de garantia de emprego para todos os adultos aptos ao trabalho e combate ao trabalho análogo à escravidão.</t>
+          <t>O programa propõe o fim imediato da escala 6x1 e a redução da jornada de trabalho para 30 horas semanais sem redução salarial, além de aumento de 100% do salário mínimo. Defende a revogação das reformas trabalhista e previdenciária e o fim da terceirização irrestrita, com regulamentação rigorosa do trabalho por aplicativos, garantindo remuneração mínima e proteção previdenciária. Propõe a criação de frentes de trabalho emergenciais, com empregos públicos diretos em obras de infraestrutura, moradia e saneamento, além de garantia de emprego para todos os adultos aptos ao trabalho e combate ao trabalho análogo à escravidão.</t>
         </is>
       </c>
       <c r="F143" s="4" t="inlineStr">

</xml_diff>